<commit_message>
Archivo roles y permisos listo
</commit_message>
<xml_diff>
--- a/DiccionarioDatos.xlsx
+++ b/DiccionarioDatos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Documents\USCO\8Semestre\IntegradorIII\documentacionDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{863095C1-0EC0-4A1E-A365-CA9D7FBBF6D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18605A5B-BF34-4216-AB70-CA95D2846D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1930" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1931" uniqueCount="483">
   <si>
     <t>Tabla</t>
   </si>
@@ -29524,7 +29524,9 @@
       <c r="B41" s="29" t="s">
         <v>480</v>
       </c>
-      <c r="C41" s="10"/>
+      <c r="C41" s="29" t="s">
+        <v>150</v>
+      </c>
       <c r="D41" s="11" t="s">
         <v>123</v>
       </c>

</xml_diff>

<commit_message>
Ultimas modificaciones de documenatacion
</commit_message>
<xml_diff>
--- a/DiccionarioDatos.xlsx
+++ b/DiccionarioDatos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Documents\USCO\8Semestre\IntegradorIII\documentacionDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18605A5B-BF34-4216-AB70-CA95D2846D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{48368241-5D3B-4CE5-BC01-8C66EA48A816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,11 +23,12 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Modulo1!$A$1:$I$1001</definedName>
   </definedNames>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1931" uniqueCount="483">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1958" uniqueCount="489">
   <si>
     <t>Tabla</t>
   </si>
@@ -1493,6 +1494,24 @@
   <si>
     <t>Identificador de la cuenta usuario.</t>
   </si>
+  <si>
+    <t>id_cuenta_usuario</t>
+  </si>
+  <si>
+    <t>uq_usuario</t>
+  </si>
+  <si>
+    <t>fk_estado_cuenta</t>
+  </si>
+  <si>
+    <t>Identificador único de la sesion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identificador único del usuario </t>
+  </si>
+  <si>
+    <t>Identificador único del estado cuenta</t>
+  </si>
 </sst>
 </file>
 
@@ -1722,22 +1741,6 @@
       </font>
     </dxf>
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF6F8F9"/>
@@ -1921,37 +1924,53 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
-  <tableStyles count="5">
+  <tableStyles count="5" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Modulos-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="17"/>
-      <tableStyleElement type="headerRow" dxfId="20"/>
-      <tableStyleElement type="firstRowStripe" dxfId="19"/>
-      <tableStyleElement type="secondRowStripe" dxfId="18"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="20"/>
+      <tableStyleElement type="headerRow" dxfId="19"/>
+      <tableStyleElement type="firstRowStripe" dxfId="18"/>
+      <tableStyleElement type="secondRowStripe" dxfId="17"/>
     </tableStyle>
     <tableStyle name="Modulo1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="13"/>
-      <tableStyleElement type="headerRow" dxfId="16"/>
-      <tableStyleElement type="firstRowStripe" dxfId="15"/>
-      <tableStyleElement type="secondRowStripe" dxfId="14"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="16"/>
+      <tableStyleElement type="headerRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="secondRowStripe" dxfId="13"/>
     </tableStyle>
     <tableStyle name="Modulo 9-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF02000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="9"/>
-      <tableStyleElement type="headerRow" dxfId="12"/>
-      <tableStyleElement type="firstRowStripe" dxfId="11"/>
-      <tableStyleElement type="secondRowStripe" dxfId="10"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="12"/>
+      <tableStyleElement type="headerRow" dxfId="11"/>
+      <tableStyleElement type="firstRowStripe" dxfId="10"/>
+      <tableStyleElement type="secondRowStripe" dxfId="9"/>
     </tableStyle>
     <tableStyle name="Modulo 2-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF03000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="5"/>
-      <tableStyleElement type="headerRow" dxfId="8"/>
-      <tableStyleElement type="firstRowStripe" dxfId="7"/>
-      <tableStyleElement type="secondRowStripe" dxfId="6"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="8"/>
+      <tableStyleElement type="headerRow" dxfId="7"/>
+      <tableStyleElement type="firstRowStripe" dxfId="6"/>
+      <tableStyleElement type="secondRowStripe" dxfId="5"/>
     </tableStyle>
     <tableStyle name="ENUMS-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF04000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="1"/>
-      <tableStyleElement type="headerRow" dxfId="4"/>
-      <tableStyleElement type="firstRowStripe" dxfId="3"/>
-      <tableStyleElement type="secondRowStripe" dxfId="2"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="4"/>
+      <tableStyleElement type="headerRow" dxfId="3"/>
+      <tableStyleElement type="firstRowStripe" dxfId="2"/>
+      <tableStyleElement type="secondRowStripe" dxfId="1"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1963,10 +1982,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -28352,7 +28367,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:I1000"/>
+  <dimension ref="A1:I1001"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="8" width="22.6640625" customWidth="1"/>
@@ -30243,260 +30258,335 @@
       </c>
     </row>
     <row r="66" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D66" s="11"/>
-      <c r="I66" s="6"/>
+      <c r="A66" t="s">
+        <v>475</v>
+      </c>
+      <c r="B66" t="s">
+        <v>483</v>
+      </c>
+      <c r="C66" t="s">
+        <v>122</v>
+      </c>
+      <c r="D66" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E66" t="s">
+        <v>124</v>
+      </c>
+      <c r="F66" t="s">
+        <v>125</v>
+      </c>
+      <c r="G66" t="s">
+        <v>124</v>
+      </c>
+      <c r="H66" t="s">
+        <v>125</v>
+      </c>
+      <c r="I66" s="7" t="s">
+        <v>486</v>
+      </c>
     </row>
     <row r="67" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D67" s="11"/>
-      <c r="I67" s="6"/>
+      <c r="A67" t="s">
+        <v>475</v>
+      </c>
+      <c r="B67" t="s">
+        <v>484</v>
+      </c>
+      <c r="C67" t="s">
+        <v>150</v>
+      </c>
+      <c r="D67" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E67" t="s">
+        <v>124</v>
+      </c>
+      <c r="F67" t="s">
+        <v>124</v>
+      </c>
+      <c r="G67" t="s">
+        <v>125</v>
+      </c>
+      <c r="H67" t="s">
+        <v>125</v>
+      </c>
+      <c r="I67" s="7" t="s">
+        <v>487</v>
+      </c>
     </row>
     <row r="68" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D68" s="11"/>
-      <c r="I68" s="6"/>
+      <c r="A68" t="s">
+        <v>475</v>
+      </c>
+      <c r="B68" t="s">
+        <v>485</v>
+      </c>
+      <c r="C68" t="s">
+        <v>150</v>
+      </c>
+      <c r="D68" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="E68" t="s">
+        <v>124</v>
+      </c>
+      <c r="F68" t="s">
+        <v>124</v>
+      </c>
+      <c r="G68" t="s">
+        <v>125</v>
+      </c>
+      <c r="H68" t="s">
+        <v>124</v>
+      </c>
+      <c r="I68" s="7" t="s">
+        <v>488</v>
+      </c>
     </row>
     <row r="69" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D69" s="11"/>
-      <c r="I69" s="6"/>
+      <c r="I69" s="7"/>
     </row>
     <row r="70" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D70" s="11"/>
-      <c r="I70" s="6"/>
+      <c r="I70" s="7"/>
     </row>
     <row r="71" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D71" s="11"/>
-      <c r="I71" s="6"/>
+      <c r="I71" s="7"/>
     </row>
     <row r="72" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D72" s="11"/>
-      <c r="I72" s="6"/>
+      <c r="I72" s="7"/>
     </row>
     <row r="73" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D73" s="11"/>
-      <c r="I73" s="6"/>
+      <c r="I73" s="7"/>
     </row>
     <row r="74" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D74" s="11"/>
-      <c r="I74" s="6"/>
+      <c r="I74" s="7"/>
     </row>
     <row r="75" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D75" s="11"/>
-      <c r="I75" s="6"/>
+      <c r="I75" s="7"/>
     </row>
     <row r="76" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D76" s="11"/>
-      <c r="I76" s="6"/>
+      <c r="I76" s="7"/>
     </row>
     <row r="77" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D77" s="11"/>
-      <c r="I77" s="6"/>
+      <c r="I77" s="7"/>
     </row>
     <row r="78" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D78" s="11"/>
-      <c r="I78" s="6"/>
+      <c r="I78" s="7"/>
     </row>
     <row r="79" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D79" s="11"/>
-      <c r="I79" s="6"/>
+      <c r="I79" s="7"/>
     </row>
     <row r="80" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D80" s="11"/>
-      <c r="I80" s="6"/>
+      <c r="I80" s="7"/>
     </row>
     <row r="81" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D81" s="11"/>
-      <c r="I81" s="6"/>
+      <c r="I81" s="7"/>
     </row>
     <row r="82" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D82" s="11"/>
-      <c r="I82" s="6"/>
+      <c r="I82" s="7"/>
     </row>
     <row r="83" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D83" s="11"/>
-      <c r="I83" s="6"/>
+      <c r="I83" s="7"/>
     </row>
     <row r="84" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D84" s="11"/>
-      <c r="I84" s="6"/>
+      <c r="I84" s="7"/>
     </row>
     <row r="85" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D85" s="11"/>
-      <c r="I85" s="6"/>
+      <c r="I85" s="7"/>
     </row>
     <row r="86" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D86" s="11"/>
-      <c r="I86" s="6"/>
+      <c r="I86" s="7"/>
     </row>
     <row r="87" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D87" s="11"/>
-      <c r="I87" s="6"/>
+      <c r="I87" s="7"/>
     </row>
     <row r="88" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D88" s="11"/>
-      <c r="I88" s="6"/>
+      <c r="I88" s="7"/>
     </row>
     <row r="89" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D89" s="11"/>
-      <c r="I89" s="6"/>
+      <c r="I89" s="7"/>
     </row>
     <row r="90" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D90" s="11"/>
-      <c r="I90" s="6"/>
+      <c r="I90" s="7"/>
     </row>
     <row r="91" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D91" s="11"/>
-      <c r="I91" s="6"/>
+      <c r="I91" s="7"/>
     </row>
     <row r="92" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D92" s="11"/>
-      <c r="I92" s="6"/>
+      <c r="I92" s="7"/>
     </row>
     <row r="93" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D93" s="11"/>
-      <c r="I93" s="6"/>
+      <c r="I93" s="7"/>
     </row>
     <row r="94" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D94" s="11"/>
-      <c r="I94" s="6"/>
+      <c r="I94" s="7"/>
     </row>
     <row r="95" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D95" s="11"/>
-      <c r="I95" s="6"/>
+      <c r="I95" s="7"/>
     </row>
     <row r="96" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D96" s="11"/>
-      <c r="I96" s="6"/>
+      <c r="I96" s="7"/>
     </row>
     <row r="97" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D97" s="11"/>
-      <c r="I97" s="6"/>
+      <c r="I97" s="7"/>
     </row>
     <row r="98" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D98" s="11"/>
-      <c r="I98" s="6"/>
+      <c r="I98" s="7"/>
     </row>
     <row r="99" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D99" s="11"/>
-      <c r="I99" s="6"/>
+      <c r="I99" s="7"/>
     </row>
     <row r="100" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D100" s="11"/>
-      <c r="I100" s="6"/>
+      <c r="I100" s="7"/>
     </row>
     <row r="101" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D101" s="11"/>
-      <c r="I101" s="6"/>
+      <c r="I101" s="7"/>
     </row>
     <row r="102" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D102" s="11"/>
-      <c r="I102" s="6"/>
+      <c r="I102" s="7"/>
     </row>
     <row r="103" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D103" s="11"/>
-      <c r="I103" s="6"/>
+      <c r="I103" s="7"/>
     </row>
     <row r="104" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D104" s="11"/>
-      <c r="I104" s="6"/>
+      <c r="I104" s="7"/>
     </row>
     <row r="105" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D105" s="11"/>
-      <c r="I105" s="6"/>
+      <c r="I105" s="7"/>
     </row>
     <row r="106" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D106" s="11"/>
-      <c r="I106" s="6"/>
+      <c r="I106" s="7"/>
     </row>
     <row r="107" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D107" s="11"/>
-      <c r="I107" s="6"/>
+      <c r="I107" s="7"/>
     </row>
     <row r="108" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D108" s="11"/>
-      <c r="I108" s="6"/>
+      <c r="I108" s="7"/>
     </row>
     <row r="109" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D109" s="11"/>
-      <c r="I109" s="6"/>
+      <c r="I109" s="7"/>
     </row>
     <row r="110" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D110" s="11"/>
-      <c r="I110" s="6"/>
+      <c r="I110" s="7"/>
     </row>
     <row r="111" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D111" s="11"/>
-      <c r="I111" s="6"/>
+      <c r="I111" s="7"/>
     </row>
     <row r="112" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D112" s="11"/>
-      <c r="I112" s="6"/>
+      <c r="I112" s="7"/>
     </row>
     <row r="113" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D113" s="11"/>
-      <c r="I113" s="6"/>
+      <c r="I113" s="7"/>
     </row>
     <row r="114" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D114" s="11"/>
-      <c r="I114" s="6"/>
+      <c r="I114" s="7"/>
     </row>
     <row r="115" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D115" s="11"/>
-      <c r="I115" s="6"/>
+      <c r="I115" s="7"/>
     </row>
     <row r="116" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D116" s="11"/>
-      <c r="I116" s="6"/>
+      <c r="I116" s="7"/>
     </row>
     <row r="117" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D117" s="11"/>
-      <c r="I117" s="6"/>
+      <c r="I117" s="7"/>
     </row>
     <row r="118" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D118" s="11"/>
-      <c r="I118" s="6"/>
+      <c r="I118" s="7"/>
     </row>
     <row r="119" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D119" s="11"/>
-      <c r="I119" s="6"/>
+      <c r="I119" s="7"/>
     </row>
     <row r="120" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D120" s="11"/>
-      <c r="I120" s="6"/>
+      <c r="I120" s="7"/>
     </row>
     <row r="121" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D121" s="11"/>
-      <c r="I121" s="6"/>
+      <c r="I121" s="7"/>
     </row>
     <row r="122" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D122" s="11"/>
-      <c r="I122" s="6"/>
+      <c r="I122" s="7"/>
     </row>
     <row r="123" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D123" s="11"/>
-      <c r="I123" s="6"/>
+      <c r="I123" s="7"/>
     </row>
     <row r="124" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D124" s="11"/>
-      <c r="I124" s="6"/>
+      <c r="I124" s="7"/>
     </row>
     <row r="125" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D125" s="11"/>
-      <c r="I125" s="6"/>
+      <c r="I125" s="7"/>
     </row>
     <row r="126" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D126" s="11"/>
-      <c r="I126" s="6"/>
+      <c r="I126" s="7"/>
     </row>
     <row r="127" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D127" s="11"/>
-      <c r="I127" s="6"/>
+      <c r="I127" s="7"/>
     </row>
     <row r="128" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D128" s="11"/>
-      <c r="I128" s="6"/>
+      <c r="I128" s="7"/>
     </row>
     <row r="129" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D129" s="11"/>
-      <c r="I129" s="6"/>
+      <c r="I129" s="7"/>
     </row>
     <row r="130" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C130" s="14" t="s">
@@ -30507,3483 +30597,3486 @@
     </row>
     <row r="131" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D131" s="11"/>
-      <c r="I131" s="6"/>
+      <c r="I131" s="7"/>
     </row>
     <row r="132" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D132" s="11"/>
-      <c r="I132" s="6"/>
+      <c r="I132" s="7"/>
     </row>
     <row r="133" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D133" s="11"/>
-      <c r="I133" s="6"/>
+      <c r="I133" s="7"/>
     </row>
     <row r="134" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D134" s="11"/>
-      <c r="I134" s="6"/>
+      <c r="I134" s="7"/>
     </row>
     <row r="135" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D135" s="11"/>
-      <c r="I135" s="6"/>
+      <c r="I135" s="7"/>
     </row>
     <row r="136" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D136" s="11"/>
-      <c r="I136" s="6"/>
+      <c r="I136" s="7"/>
     </row>
     <row r="137" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D137" s="11"/>
-      <c r="I137" s="6"/>
+      <c r="I137" s="7"/>
     </row>
     <row r="138" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D138" s="11"/>
-      <c r="I138" s="6"/>
+      <c r="I138" s="7"/>
     </row>
     <row r="139" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D139" s="11"/>
-      <c r="I139" s="6"/>
+      <c r="I139" s="7"/>
     </row>
     <row r="140" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D140" s="11"/>
-      <c r="I140" s="6"/>
+      <c r="I140" s="7"/>
     </row>
     <row r="141" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D141" s="11"/>
-      <c r="I141" s="6"/>
+      <c r="I141" s="7"/>
     </row>
     <row r="142" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D142" s="11"/>
-      <c r="I142" s="6"/>
+      <c r="I142" s="7"/>
     </row>
     <row r="143" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D143" s="11"/>
-      <c r="I143" s="6"/>
+      <c r="I143" s="7"/>
     </row>
     <row r="144" spans="3:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D144" s="11"/>
-      <c r="I144" s="6"/>
+      <c r="I144" s="7"/>
     </row>
     <row r="145" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D145" s="11"/>
-      <c r="I145" s="6"/>
+      <c r="I145" s="7"/>
     </row>
     <row r="146" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D146" s="11"/>
-      <c r="I146" s="6"/>
+      <c r="I146" s="7"/>
     </row>
     <row r="147" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D147" s="11"/>
-      <c r="I147" s="6"/>
+      <c r="I147" s="7"/>
     </row>
     <row r="148" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D148" s="11"/>
-      <c r="I148" s="6"/>
+      <c r="I148" s="7"/>
     </row>
     <row r="149" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D149" s="11"/>
-      <c r="I149" s="6"/>
+      <c r="I149" s="7"/>
     </row>
     <row r="150" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D150" s="11"/>
-      <c r="I150" s="6"/>
+      <c r="I150" s="7"/>
     </row>
     <row r="151" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D151" s="11"/>
-      <c r="I151" s="6"/>
+      <c r="I151" s="7"/>
     </row>
     <row r="152" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D152" s="11"/>
-      <c r="I152" s="6"/>
+      <c r="I152" s="7"/>
     </row>
     <row r="153" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D153" s="11"/>
-      <c r="I153" s="6"/>
+      <c r="I153" s="7"/>
     </row>
     <row r="154" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D154" s="11"/>
-      <c r="I154" s="6"/>
+      <c r="I154" s="7"/>
     </row>
     <row r="155" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D155" s="11"/>
-      <c r="I155" s="6"/>
+      <c r="I155" s="7"/>
     </row>
     <row r="156" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D156" s="11"/>
-      <c r="I156" s="6"/>
+      <c r="I156" s="7"/>
     </row>
     <row r="157" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D157" s="11"/>
-      <c r="I157" s="6"/>
+      <c r="I157" s="7"/>
     </row>
     <row r="158" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D158" s="11"/>
-      <c r="I158" s="6"/>
+      <c r="I158" s="7"/>
     </row>
     <row r="159" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D159" s="11"/>
-      <c r="I159" s="6"/>
+      <c r="I159" s="7"/>
     </row>
     <row r="160" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D160" s="11"/>
-      <c r="I160" s="6"/>
+      <c r="I160" s="7"/>
     </row>
     <row r="161" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D161" s="11"/>
-      <c r="I161" s="6"/>
+      <c r="I161" s="7"/>
     </row>
     <row r="162" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D162" s="11"/>
-      <c r="I162" s="6"/>
+      <c r="I162" s="7"/>
     </row>
     <row r="163" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D163" s="11"/>
-      <c r="I163" s="6"/>
+      <c r="I163" s="7"/>
     </row>
     <row r="164" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D164" s="11"/>
-      <c r="I164" s="6"/>
+      <c r="I164" s="7"/>
     </row>
     <row r="165" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D165" s="11"/>
-      <c r="I165" s="6"/>
+      <c r="I165" s="7"/>
     </row>
     <row r="166" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D166" s="11"/>
-      <c r="I166" s="6"/>
+      <c r="I166" s="7"/>
     </row>
     <row r="167" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D167" s="11"/>
-      <c r="I167" s="6"/>
+      <c r="I167" s="7"/>
     </row>
     <row r="168" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D168" s="11"/>
-      <c r="I168" s="6"/>
+      <c r="I168" s="7"/>
     </row>
     <row r="169" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D169" s="11"/>
-      <c r="I169" s="6"/>
+      <c r="I169" s="7"/>
     </row>
     <row r="170" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D170" s="11"/>
-      <c r="I170" s="6"/>
+      <c r="I170" s="7"/>
     </row>
     <row r="171" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D171" s="11"/>
-      <c r="I171" s="6"/>
+      <c r="I171" s="7"/>
     </row>
     <row r="172" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D172" s="11"/>
-      <c r="I172" s="6"/>
+      <c r="I172" s="7"/>
     </row>
     <row r="173" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D173" s="11"/>
-      <c r="I173" s="6"/>
+      <c r="I173" s="7"/>
     </row>
     <row r="174" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D174" s="11"/>
-      <c r="I174" s="6"/>
+      <c r="I174" s="7"/>
     </row>
     <row r="175" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D175" s="11"/>
-      <c r="I175" s="6"/>
+      <c r="I175" s="7"/>
     </row>
     <row r="176" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D176" s="11"/>
-      <c r="I176" s="6"/>
+      <c r="I176" s="7"/>
     </row>
     <row r="177" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D177" s="11"/>
-      <c r="I177" s="6"/>
+      <c r="I177" s="7"/>
     </row>
     <row r="178" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D178" s="11"/>
-      <c r="I178" s="6"/>
+      <c r="I178" s="7"/>
     </row>
     <row r="179" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D179" s="11"/>
-      <c r="I179" s="6"/>
+      <c r="I179" s="7"/>
     </row>
     <row r="180" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D180" s="11"/>
-      <c r="I180" s="6"/>
+      <c r="I180" s="7"/>
     </row>
     <row r="181" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D181" s="11"/>
-      <c r="I181" s="6"/>
+      <c r="I181" s="7"/>
     </row>
     <row r="182" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D182" s="11"/>
-      <c r="I182" s="6"/>
+      <c r="I182" s="7"/>
     </row>
     <row r="183" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D183" s="11"/>
-      <c r="I183" s="6"/>
+      <c r="I183" s="7"/>
     </row>
     <row r="184" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D184" s="11"/>
-      <c r="I184" s="6"/>
+      <c r="I184" s="7"/>
     </row>
     <row r="185" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D185" s="11"/>
-      <c r="I185" s="6"/>
+      <c r="I185" s="7"/>
     </row>
     <row r="186" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D186" s="11"/>
-      <c r="I186" s="6"/>
+      <c r="I186" s="7"/>
     </row>
     <row r="187" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D187" s="11"/>
-      <c r="I187" s="6"/>
+      <c r="I187" s="7"/>
     </row>
     <row r="188" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D188" s="11"/>
-      <c r="I188" s="6"/>
+      <c r="I188" s="7"/>
     </row>
     <row r="189" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D189" s="11"/>
-      <c r="I189" s="6"/>
+      <c r="I189" s="7"/>
     </row>
     <row r="190" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D190" s="11"/>
-      <c r="I190" s="6"/>
+      <c r="I190" s="7"/>
     </row>
     <row r="191" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D191" s="11"/>
-      <c r="I191" s="6"/>
+      <c r="I191" s="7"/>
     </row>
     <row r="192" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D192" s="11"/>
-      <c r="I192" s="6"/>
+      <c r="I192" s="7"/>
     </row>
     <row r="193" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D193" s="11"/>
-      <c r="I193" s="6"/>
+      <c r="I193" s="7"/>
     </row>
     <row r="194" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D194" s="11"/>
-      <c r="I194" s="6"/>
+      <c r="I194" s="7"/>
     </row>
     <row r="195" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D195" s="11"/>
-      <c r="I195" s="6"/>
+      <c r="I195" s="7"/>
     </row>
     <row r="196" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D196" s="11"/>
-      <c r="I196" s="6"/>
+      <c r="I196" s="7"/>
     </row>
     <row r="197" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D197" s="11"/>
-      <c r="I197" s="6"/>
+      <c r="I197" s="7"/>
     </row>
     <row r="198" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D198" s="11"/>
-      <c r="I198" s="6"/>
+      <c r="I198" s="7"/>
     </row>
     <row r="199" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D199" s="11"/>
-      <c r="I199" s="6"/>
+      <c r="I199" s="7"/>
     </row>
     <row r="200" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D200" s="11"/>
-      <c r="I200" s="6"/>
+      <c r="I200" s="7"/>
     </row>
     <row r="201" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D201" s="11"/>
-      <c r="I201" s="6"/>
+      <c r="I201" s="7"/>
     </row>
     <row r="202" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D202" s="11"/>
-      <c r="I202" s="6"/>
+      <c r="I202" s="7"/>
     </row>
     <row r="203" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D203" s="11"/>
-      <c r="I203" s="6"/>
+      <c r="I203" s="7"/>
     </row>
     <row r="204" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D204" s="11"/>
-      <c r="I204" s="6"/>
+      <c r="I204" s="7"/>
     </row>
     <row r="205" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D205" s="11"/>
-      <c r="I205" s="6"/>
+      <c r="I205" s="7"/>
     </row>
     <row r="206" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D206" s="11"/>
-      <c r="I206" s="6"/>
+      <c r="I206" s="7"/>
     </row>
     <row r="207" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D207" s="11"/>
-      <c r="I207" s="6"/>
+      <c r="I207" s="7"/>
     </row>
     <row r="208" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D208" s="11"/>
-      <c r="I208" s="6"/>
+      <c r="I208" s="7"/>
     </row>
     <row r="209" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D209" s="11"/>
-      <c r="I209" s="6"/>
+      <c r="I209" s="7"/>
     </row>
     <row r="210" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D210" s="11"/>
-      <c r="I210" s="6"/>
+      <c r="I210" s="7"/>
     </row>
     <row r="211" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D211" s="11"/>
-      <c r="I211" s="6"/>
+      <c r="I211" s="7"/>
     </row>
     <row r="212" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D212" s="11"/>
-      <c r="I212" s="6"/>
+      <c r="I212" s="7"/>
     </row>
     <row r="213" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D213" s="11"/>
-      <c r="I213" s="6"/>
+      <c r="I213" s="7"/>
     </row>
     <row r="214" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D214" s="11"/>
-      <c r="I214" s="6"/>
+      <c r="I214" s="7"/>
     </row>
     <row r="215" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D215" s="11"/>
-      <c r="I215" s="6"/>
+      <c r="I215" s="7"/>
     </row>
     <row r="216" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D216" s="11"/>
-      <c r="I216" s="6"/>
+      <c r="I216" s="7"/>
     </row>
     <row r="217" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D217" s="11"/>
-      <c r="I217" s="6"/>
+      <c r="I217" s="7"/>
     </row>
     <row r="218" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D218" s="11"/>
-      <c r="I218" s="6"/>
+      <c r="I218" s="7"/>
     </row>
     <row r="219" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D219" s="11"/>
-      <c r="I219" s="6"/>
+      <c r="I219" s="7"/>
     </row>
     <row r="220" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D220" s="11"/>
-      <c r="I220" s="6"/>
+      <c r="I220" s="7"/>
     </row>
     <row r="221" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D221" s="11"/>
-      <c r="I221" s="6"/>
+      <c r="I221" s="7"/>
     </row>
     <row r="222" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D222" s="11"/>
-      <c r="I222" s="6"/>
+      <c r="I222" s="7"/>
     </row>
     <row r="223" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D223" s="11"/>
-      <c r="I223" s="6"/>
+      <c r="I223" s="7"/>
     </row>
     <row r="224" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D224" s="11"/>
-      <c r="I224" s="6"/>
+      <c r="I224" s="7"/>
     </row>
     <row r="225" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D225" s="11"/>
-      <c r="I225" s="6"/>
+      <c r="I225" s="7"/>
     </row>
     <row r="226" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D226" s="11"/>
-      <c r="I226" s="6"/>
+      <c r="I226" s="7"/>
     </row>
     <row r="227" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D227" s="11"/>
-      <c r="I227" s="6"/>
+      <c r="I227" s="7"/>
     </row>
     <row r="228" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D228" s="11"/>
-      <c r="I228" s="6"/>
+      <c r="I228" s="7"/>
     </row>
     <row r="229" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D229" s="11"/>
-      <c r="I229" s="6"/>
+      <c r="I229" s="7"/>
     </row>
     <row r="230" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D230" s="11"/>
-      <c r="I230" s="6"/>
+      <c r="I230" s="7"/>
     </row>
     <row r="231" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D231" s="11"/>
-      <c r="I231" s="6"/>
+      <c r="I231" s="7"/>
     </row>
     <row r="232" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D232" s="11"/>
-      <c r="I232" s="6"/>
+      <c r="I232" s="7"/>
     </row>
     <row r="233" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D233" s="11"/>
-      <c r="I233" s="6"/>
+      <c r="I233" s="7"/>
     </row>
     <row r="234" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D234" s="11"/>
-      <c r="I234" s="6"/>
+      <c r="I234" s="7"/>
     </row>
     <row r="235" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D235" s="11"/>
-      <c r="I235" s="6"/>
+      <c r="I235" s="7"/>
     </row>
     <row r="236" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D236" s="11"/>
-      <c r="I236" s="6"/>
+      <c r="I236" s="7"/>
     </row>
     <row r="237" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D237" s="11"/>
-      <c r="I237" s="6"/>
+      <c r="I237" s="7"/>
     </row>
     <row r="238" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D238" s="11"/>
-      <c r="I238" s="6"/>
+      <c r="I238" s="7"/>
     </row>
     <row r="239" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D239" s="11"/>
-      <c r="I239" s="6"/>
+      <c r="I239" s="7"/>
     </row>
     <row r="240" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D240" s="11"/>
-      <c r="I240" s="6"/>
+      <c r="I240" s="7"/>
     </row>
     <row r="241" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D241" s="11"/>
-      <c r="I241" s="6"/>
+      <c r="I241" s="7"/>
     </row>
     <row r="242" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D242" s="11"/>
-      <c r="I242" s="6"/>
+      <c r="I242" s="7"/>
     </row>
     <row r="243" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D243" s="11"/>
-      <c r="I243" s="6"/>
+      <c r="I243" s="7"/>
     </row>
     <row r="244" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D244" s="11"/>
-      <c r="I244" s="6"/>
+      <c r="I244" s="7"/>
     </row>
     <row r="245" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D245" s="11"/>
-      <c r="I245" s="6"/>
+      <c r="I245" s="7"/>
     </row>
     <row r="246" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D246" s="11"/>
-      <c r="I246" s="6"/>
+      <c r="I246" s="7"/>
     </row>
     <row r="247" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D247" s="11"/>
-      <c r="I247" s="6"/>
+      <c r="I247" s="7"/>
     </row>
     <row r="248" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D248" s="11"/>
-      <c r="I248" s="6"/>
+      <c r="I248" s="7"/>
     </row>
     <row r="249" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D249" s="11"/>
-      <c r="I249" s="6"/>
+      <c r="I249" s="7"/>
     </row>
     <row r="250" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D250" s="11"/>
-      <c r="I250" s="6"/>
+      <c r="I250" s="7"/>
     </row>
     <row r="251" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D251" s="11"/>
-      <c r="I251" s="6"/>
+      <c r="I251" s="7"/>
     </row>
     <row r="252" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D252" s="11"/>
-      <c r="I252" s="6"/>
+      <c r="I252" s="7"/>
     </row>
     <row r="253" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D253" s="11"/>
-      <c r="I253" s="6"/>
+      <c r="I253" s="7"/>
     </row>
     <row r="254" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D254" s="11"/>
-      <c r="I254" s="6"/>
+      <c r="I254" s="7"/>
     </row>
     <row r="255" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D255" s="11"/>
-      <c r="I255" s="6"/>
+      <c r="I255" s="7"/>
     </row>
     <row r="256" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D256" s="11"/>
-      <c r="I256" s="6"/>
+      <c r="I256" s="7"/>
     </row>
     <row r="257" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D257" s="11"/>
-      <c r="I257" s="6"/>
+      <c r="I257" s="7"/>
     </row>
     <row r="258" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D258" s="11"/>
-      <c r="I258" s="6"/>
+      <c r="I258" s="7"/>
     </row>
     <row r="259" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D259" s="11"/>
-      <c r="I259" s="6"/>
+      <c r="I259" s="7"/>
     </row>
     <row r="260" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D260" s="11"/>
-      <c r="I260" s="6"/>
+      <c r="I260" s="7"/>
     </row>
     <row r="261" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D261" s="11"/>
-      <c r="I261" s="6"/>
+      <c r="I261" s="7"/>
     </row>
     <row r="262" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D262" s="11"/>
-      <c r="I262" s="6"/>
+      <c r="I262" s="7"/>
     </row>
     <row r="263" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D263" s="11"/>
-      <c r="I263" s="6"/>
+      <c r="I263" s="7"/>
     </row>
     <row r="264" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D264" s="11"/>
-      <c r="I264" s="6"/>
+      <c r="I264" s="7"/>
     </row>
     <row r="265" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D265" s="11"/>
-      <c r="I265" s="6"/>
+      <c r="I265" s="7"/>
     </row>
     <row r="266" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D266" s="11"/>
-      <c r="I266" s="6"/>
+      <c r="I266" s="7"/>
     </row>
     <row r="267" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D267" s="11"/>
-      <c r="I267" s="6"/>
+      <c r="I267" s="7"/>
     </row>
     <row r="268" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D268" s="11"/>
-      <c r="I268" s="6"/>
+      <c r="I268" s="7"/>
     </row>
     <row r="269" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D269" s="11"/>
-      <c r="I269" s="6"/>
+      <c r="I269" s="7"/>
     </row>
     <row r="270" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D270" s="11"/>
-      <c r="I270" s="6"/>
+      <c r="I270" s="7"/>
     </row>
     <row r="271" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D271" s="11"/>
-      <c r="I271" s="6"/>
+      <c r="I271" s="7"/>
     </row>
     <row r="272" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D272" s="11"/>
-      <c r="I272" s="6"/>
+      <c r="I272" s="7"/>
     </row>
     <row r="273" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D273" s="11"/>
-      <c r="I273" s="6"/>
+      <c r="I273" s="7"/>
     </row>
     <row r="274" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D274" s="11"/>
-      <c r="I274" s="6"/>
+      <c r="I274" s="7"/>
     </row>
     <row r="275" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D275" s="11"/>
-      <c r="I275" s="6"/>
+      <c r="I275" s="7"/>
     </row>
     <row r="276" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D276" s="11"/>
-      <c r="I276" s="6"/>
+      <c r="I276" s="7"/>
     </row>
     <row r="277" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D277" s="11"/>
-      <c r="I277" s="6"/>
+      <c r="I277" s="7"/>
     </row>
     <row r="278" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D278" s="11"/>
-      <c r="I278" s="6"/>
+      <c r="I278" s="7"/>
     </row>
     <row r="279" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D279" s="11"/>
-      <c r="I279" s="6"/>
+      <c r="I279" s="7"/>
     </row>
     <row r="280" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D280" s="11"/>
-      <c r="I280" s="6"/>
+      <c r="I280" s="7"/>
     </row>
     <row r="281" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D281" s="11"/>
-      <c r="I281" s="6"/>
+      <c r="I281" s="7"/>
     </row>
     <row r="282" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D282" s="11"/>
-      <c r="I282" s="6"/>
+      <c r="I282" s="7"/>
     </row>
     <row r="283" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D283" s="11"/>
-      <c r="I283" s="6"/>
+      <c r="I283" s="7"/>
     </row>
     <row r="284" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D284" s="11"/>
-      <c r="I284" s="6"/>
+      <c r="I284" s="7"/>
     </row>
     <row r="285" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D285" s="11"/>
-      <c r="I285" s="6"/>
+      <c r="I285" s="7"/>
     </row>
     <row r="286" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D286" s="11"/>
-      <c r="I286" s="6"/>
+      <c r="I286" s="7"/>
     </row>
     <row r="287" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D287" s="11"/>
-      <c r="I287" s="6"/>
+      <c r="I287" s="7"/>
     </row>
     <row r="288" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D288" s="11"/>
-      <c r="I288" s="6"/>
+      <c r="I288" s="7"/>
     </row>
     <row r="289" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D289" s="11"/>
-      <c r="I289" s="6"/>
+      <c r="I289" s="7"/>
     </row>
     <row r="290" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D290" s="11"/>
-      <c r="I290" s="6"/>
+      <c r="I290" s="7"/>
     </row>
     <row r="291" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D291" s="11"/>
-      <c r="I291" s="6"/>
+      <c r="I291" s="7"/>
     </row>
     <row r="292" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D292" s="11"/>
-      <c r="I292" s="6"/>
+      <c r="I292" s="7"/>
     </row>
     <row r="293" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D293" s="11"/>
-      <c r="I293" s="6"/>
+      <c r="I293" s="7"/>
     </row>
     <row r="294" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D294" s="11"/>
-      <c r="I294" s="6"/>
+      <c r="I294" s="7"/>
     </row>
     <row r="295" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D295" s="11"/>
-      <c r="I295" s="6"/>
+      <c r="I295" s="7"/>
     </row>
     <row r="296" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D296" s="11"/>
-      <c r="I296" s="6"/>
+      <c r="I296" s="7"/>
     </row>
     <row r="297" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D297" s="11"/>
-      <c r="I297" s="6"/>
+      <c r="I297" s="7"/>
     </row>
     <row r="298" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D298" s="11"/>
-      <c r="I298" s="6"/>
+      <c r="I298" s="7"/>
     </row>
     <row r="299" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D299" s="11"/>
-      <c r="I299" s="6"/>
+      <c r="I299" s="7"/>
     </row>
     <row r="300" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D300" s="11"/>
-      <c r="I300" s="6"/>
+      <c r="I300" s="7"/>
     </row>
     <row r="301" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D301" s="11"/>
-      <c r="I301" s="6"/>
+      <c r="I301" s="7"/>
     </row>
     <row r="302" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D302" s="11"/>
-      <c r="I302" s="6"/>
+      <c r="I302" s="7"/>
     </row>
     <row r="303" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D303" s="11"/>
-      <c r="I303" s="6"/>
+      <c r="I303" s="7"/>
     </row>
     <row r="304" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D304" s="11"/>
-      <c r="I304" s="6"/>
+      <c r="I304" s="7"/>
     </row>
     <row r="305" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D305" s="11"/>
-      <c r="I305" s="6"/>
+      <c r="I305" s="7"/>
     </row>
     <row r="306" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D306" s="11"/>
-      <c r="I306" s="6"/>
+      <c r="I306" s="7"/>
     </row>
     <row r="307" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D307" s="11"/>
-      <c r="I307" s="6"/>
+      <c r="I307" s="7"/>
     </row>
     <row r="308" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D308" s="11"/>
-      <c r="I308" s="6"/>
+      <c r="I308" s="7"/>
     </row>
     <row r="309" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D309" s="11"/>
-      <c r="I309" s="6"/>
+      <c r="I309" s="7"/>
     </row>
     <row r="310" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D310" s="11"/>
-      <c r="I310" s="6"/>
+      <c r="I310" s="7"/>
     </row>
     <row r="311" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D311" s="11"/>
-      <c r="I311" s="6"/>
+      <c r="I311" s="7"/>
     </row>
     <row r="312" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D312" s="11"/>
-      <c r="I312" s="6"/>
+      <c r="I312" s="7"/>
     </row>
     <row r="313" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D313" s="11"/>
-      <c r="I313" s="6"/>
+      <c r="I313" s="7"/>
     </row>
     <row r="314" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D314" s="11"/>
-      <c r="I314" s="6"/>
+      <c r="I314" s="7"/>
     </row>
     <row r="315" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D315" s="11"/>
-      <c r="I315" s="6"/>
+      <c r="I315" s="7"/>
     </row>
     <row r="316" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D316" s="11"/>
-      <c r="I316" s="6"/>
+      <c r="I316" s="7"/>
     </row>
     <row r="317" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D317" s="11"/>
-      <c r="I317" s="6"/>
+      <c r="I317" s="7"/>
     </row>
     <row r="318" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D318" s="11"/>
-      <c r="I318" s="6"/>
+      <c r="I318" s="7"/>
     </row>
     <row r="319" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D319" s="11"/>
-      <c r="I319" s="6"/>
+      <c r="I319" s="7"/>
     </row>
     <row r="320" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D320" s="11"/>
-      <c r="I320" s="6"/>
+      <c r="I320" s="7"/>
     </row>
     <row r="321" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D321" s="11"/>
-      <c r="I321" s="6"/>
+      <c r="I321" s="7"/>
     </row>
     <row r="322" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D322" s="11"/>
-      <c r="I322" s="6"/>
+      <c r="I322" s="7"/>
     </row>
     <row r="323" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D323" s="11"/>
-      <c r="I323" s="6"/>
+      <c r="I323" s="7"/>
     </row>
     <row r="324" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D324" s="11"/>
-      <c r="I324" s="6"/>
+      <c r="I324" s="7"/>
     </row>
     <row r="325" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D325" s="11"/>
-      <c r="I325" s="6"/>
+      <c r="I325" s="7"/>
     </row>
     <row r="326" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D326" s="11"/>
-      <c r="I326" s="6"/>
+      <c r="I326" s="7"/>
     </row>
     <row r="327" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D327" s="11"/>
-      <c r="I327" s="6"/>
+      <c r="I327" s="7"/>
     </row>
     <row r="328" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D328" s="11"/>
-      <c r="I328" s="6"/>
+      <c r="I328" s="7"/>
     </row>
     <row r="329" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D329" s="11"/>
-      <c r="I329" s="6"/>
+      <c r="I329" s="7"/>
     </row>
     <row r="330" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D330" s="11"/>
-      <c r="I330" s="6"/>
+      <c r="I330" s="7"/>
     </row>
     <row r="331" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D331" s="11"/>
-      <c r="I331" s="6"/>
+      <c r="I331" s="7"/>
     </row>
     <row r="332" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D332" s="11"/>
-      <c r="I332" s="6"/>
+      <c r="I332" s="7"/>
     </row>
     <row r="333" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D333" s="11"/>
-      <c r="I333" s="6"/>
+      <c r="I333" s="7"/>
     </row>
     <row r="334" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D334" s="11"/>
-      <c r="I334" s="6"/>
+      <c r="I334" s="7"/>
     </row>
     <row r="335" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D335" s="11"/>
-      <c r="I335" s="6"/>
+      <c r="I335" s="7"/>
     </row>
     <row r="336" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D336" s="11"/>
-      <c r="I336" s="6"/>
+      <c r="I336" s="7"/>
     </row>
     <row r="337" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D337" s="11"/>
-      <c r="I337" s="6"/>
+      <c r="I337" s="7"/>
     </row>
     <row r="338" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D338" s="11"/>
-      <c r="I338" s="6"/>
+      <c r="I338" s="7"/>
     </row>
     <row r="339" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D339" s="11"/>
-      <c r="I339" s="6"/>
+      <c r="I339" s="7"/>
     </row>
     <row r="340" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D340" s="11"/>
-      <c r="I340" s="6"/>
+      <c r="I340" s="7"/>
     </row>
     <row r="341" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D341" s="11"/>
-      <c r="I341" s="6"/>
+      <c r="I341" s="7"/>
     </row>
     <row r="342" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D342" s="11"/>
-      <c r="I342" s="6"/>
+      <c r="I342" s="7"/>
     </row>
     <row r="343" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D343" s="11"/>
-      <c r="I343" s="6"/>
+      <c r="I343" s="7"/>
     </row>
     <row r="344" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D344" s="11"/>
-      <c r="I344" s="6"/>
+      <c r="I344" s="7"/>
     </row>
     <row r="345" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D345" s="11"/>
-      <c r="I345" s="6"/>
+      <c r="I345" s="7"/>
     </row>
     <row r="346" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D346" s="11"/>
-      <c r="I346" s="6"/>
+      <c r="I346" s="7"/>
     </row>
     <row r="347" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D347" s="11"/>
-      <c r="I347" s="6"/>
+      <c r="I347" s="7"/>
     </row>
     <row r="348" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D348" s="11"/>
-      <c r="I348" s="6"/>
+      <c r="I348" s="7"/>
     </row>
     <row r="349" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D349" s="11"/>
-      <c r="I349" s="6"/>
+      <c r="I349" s="7"/>
     </row>
     <row r="350" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D350" s="11"/>
-      <c r="I350" s="6"/>
+      <c r="I350" s="7"/>
     </row>
     <row r="351" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D351" s="11"/>
-      <c r="I351" s="6"/>
+      <c r="I351" s="7"/>
     </row>
     <row r="352" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D352" s="11"/>
-      <c r="I352" s="6"/>
+      <c r="I352" s="7"/>
     </row>
     <row r="353" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D353" s="11"/>
-      <c r="I353" s="6"/>
+      <c r="I353" s="7"/>
     </row>
     <row r="354" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D354" s="11"/>
-      <c r="I354" s="6"/>
+      <c r="I354" s="7"/>
     </row>
     <row r="355" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D355" s="11"/>
-      <c r="I355" s="6"/>
+      <c r="I355" s="7"/>
     </row>
     <row r="356" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D356" s="11"/>
-      <c r="I356" s="6"/>
+      <c r="I356" s="7"/>
     </row>
     <row r="357" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D357" s="11"/>
-      <c r="I357" s="6"/>
+      <c r="I357" s="7"/>
     </row>
     <row r="358" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D358" s="11"/>
-      <c r="I358" s="6"/>
+      <c r="I358" s="7"/>
     </row>
     <row r="359" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D359" s="11"/>
-      <c r="I359" s="6"/>
+      <c r="I359" s="7"/>
     </row>
     <row r="360" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D360" s="11"/>
-      <c r="I360" s="6"/>
+      <c r="I360" s="7"/>
     </row>
     <row r="361" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D361" s="11"/>
-      <c r="I361" s="6"/>
+      <c r="I361" s="7"/>
     </row>
     <row r="362" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D362" s="11"/>
-      <c r="I362" s="6"/>
+      <c r="I362" s="7"/>
     </row>
     <row r="363" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D363" s="11"/>
-      <c r="I363" s="6"/>
+      <c r="I363" s="7"/>
     </row>
     <row r="364" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D364" s="11"/>
-      <c r="I364" s="6"/>
+      <c r="I364" s="7"/>
     </row>
     <row r="365" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D365" s="11"/>
-      <c r="I365" s="6"/>
+      <c r="I365" s="7"/>
     </row>
     <row r="366" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D366" s="11"/>
-      <c r="I366" s="6"/>
+      <c r="I366" s="7"/>
     </row>
     <row r="367" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D367" s="11"/>
-      <c r="I367" s="6"/>
+      <c r="I367" s="7"/>
     </row>
     <row r="368" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D368" s="11"/>
-      <c r="I368" s="6"/>
+      <c r="I368" s="7"/>
     </row>
     <row r="369" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D369" s="11"/>
-      <c r="I369" s="6"/>
+      <c r="I369" s="7"/>
     </row>
     <row r="370" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D370" s="11"/>
-      <c r="I370" s="6"/>
+      <c r="I370" s="7"/>
     </row>
     <row r="371" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D371" s="11"/>
-      <c r="I371" s="6"/>
+      <c r="I371" s="7"/>
     </row>
     <row r="372" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D372" s="11"/>
-      <c r="I372" s="6"/>
+      <c r="I372" s="7"/>
     </row>
     <row r="373" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D373" s="11"/>
-      <c r="I373" s="6"/>
+      <c r="I373" s="7"/>
     </row>
     <row r="374" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D374" s="11"/>
-      <c r="I374" s="6"/>
+      <c r="I374" s="7"/>
     </row>
     <row r="375" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D375" s="11"/>
-      <c r="I375" s="6"/>
+      <c r="I375" s="7"/>
     </row>
     <row r="376" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D376" s="11"/>
-      <c r="I376" s="6"/>
+      <c r="I376" s="7"/>
     </row>
     <row r="377" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D377" s="11"/>
-      <c r="I377" s="6"/>
+      <c r="I377" s="7"/>
     </row>
     <row r="378" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D378" s="11"/>
-      <c r="I378" s="6"/>
+      <c r="I378" s="7"/>
     </row>
     <row r="379" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D379" s="11"/>
-      <c r="I379" s="6"/>
+      <c r="I379" s="7"/>
     </row>
     <row r="380" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D380" s="11"/>
-      <c r="I380" s="6"/>
+      <c r="I380" s="7"/>
     </row>
     <row r="381" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D381" s="11"/>
-      <c r="I381" s="6"/>
+      <c r="I381" s="7"/>
     </row>
     <row r="382" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D382" s="11"/>
-      <c r="I382" s="6"/>
+      <c r="I382" s="7"/>
     </row>
     <row r="383" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D383" s="11"/>
-      <c r="I383" s="6"/>
+      <c r="I383" s="7"/>
     </row>
     <row r="384" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D384" s="11"/>
-      <c r="I384" s="6"/>
+      <c r="I384" s="7"/>
     </row>
     <row r="385" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D385" s="11"/>
-      <c r="I385" s="6"/>
+      <c r="I385" s="7"/>
     </row>
     <row r="386" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D386" s="11"/>
-      <c r="I386" s="6"/>
+      <c r="I386" s="7"/>
     </row>
     <row r="387" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D387" s="11"/>
-      <c r="I387" s="6"/>
+      <c r="I387" s="7"/>
     </row>
     <row r="388" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D388" s="11"/>
-      <c r="I388" s="6"/>
+      <c r="I388" s="7"/>
     </row>
     <row r="389" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D389" s="11"/>
-      <c r="I389" s="6"/>
+      <c r="I389" s="7"/>
     </row>
     <row r="390" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D390" s="11"/>
-      <c r="I390" s="6"/>
+      <c r="I390" s="7"/>
     </row>
     <row r="391" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D391" s="11"/>
-      <c r="I391" s="6"/>
+      <c r="I391" s="7"/>
     </row>
     <row r="392" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D392" s="11"/>
-      <c r="I392" s="6"/>
+      <c r="I392" s="7"/>
     </row>
     <row r="393" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D393" s="11"/>
-      <c r="I393" s="6"/>
+      <c r="I393" s="7"/>
     </row>
     <row r="394" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D394" s="11"/>
-      <c r="I394" s="6"/>
+      <c r="I394" s="7"/>
     </row>
     <row r="395" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D395" s="11"/>
-      <c r="I395" s="6"/>
+      <c r="I395" s="7"/>
     </row>
     <row r="396" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D396" s="11"/>
-      <c r="I396" s="6"/>
+      <c r="I396" s="7"/>
     </row>
     <row r="397" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D397" s="11"/>
-      <c r="I397" s="6"/>
+      <c r="I397" s="7"/>
     </row>
     <row r="398" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D398" s="11"/>
-      <c r="I398" s="6"/>
+      <c r="I398" s="7"/>
     </row>
     <row r="399" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D399" s="11"/>
-      <c r="I399" s="6"/>
+      <c r="I399" s="7"/>
     </row>
     <row r="400" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D400" s="11"/>
-      <c r="I400" s="6"/>
+      <c r="I400" s="7"/>
     </row>
     <row r="401" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D401" s="11"/>
-      <c r="I401" s="6"/>
+      <c r="I401" s="7"/>
     </row>
     <row r="402" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D402" s="11"/>
-      <c r="I402" s="6"/>
+      <c r="I402" s="7"/>
     </row>
     <row r="403" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D403" s="11"/>
-      <c r="I403" s="6"/>
+      <c r="I403" s="7"/>
     </row>
     <row r="404" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D404" s="11"/>
-      <c r="I404" s="6"/>
+      <c r="I404" s="7"/>
     </row>
     <row r="405" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D405" s="11"/>
-      <c r="I405" s="6"/>
+      <c r="I405" s="7"/>
     </row>
     <row r="406" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D406" s="11"/>
-      <c r="I406" s="6"/>
+      <c r="I406" s="7"/>
     </row>
     <row r="407" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D407" s="11"/>
-      <c r="I407" s="6"/>
+      <c r="I407" s="7"/>
     </row>
     <row r="408" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D408" s="11"/>
-      <c r="I408" s="6"/>
+      <c r="I408" s="7"/>
     </row>
     <row r="409" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D409" s="11"/>
-      <c r="I409" s="6"/>
+      <c r="I409" s="7"/>
     </row>
     <row r="410" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D410" s="11"/>
-      <c r="I410" s="6"/>
+      <c r="I410" s="7"/>
     </row>
     <row r="411" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D411" s="11"/>
-      <c r="I411" s="6"/>
+      <c r="I411" s="7"/>
     </row>
     <row r="412" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D412" s="11"/>
-      <c r="I412" s="6"/>
+      <c r="I412" s="7"/>
     </row>
     <row r="413" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D413" s="11"/>
-      <c r="I413" s="6"/>
+      <c r="I413" s="7"/>
     </row>
     <row r="414" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D414" s="11"/>
-      <c r="I414" s="6"/>
+      <c r="I414" s="7"/>
     </row>
     <row r="415" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D415" s="11"/>
-      <c r="I415" s="6"/>
+      <c r="I415" s="7"/>
     </row>
     <row r="416" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D416" s="11"/>
-      <c r="I416" s="6"/>
+      <c r="I416" s="7"/>
     </row>
     <row r="417" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D417" s="11"/>
-      <c r="I417" s="6"/>
+      <c r="I417" s="7"/>
     </row>
     <row r="418" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D418" s="11"/>
-      <c r="I418" s="6"/>
+      <c r="I418" s="7"/>
     </row>
     <row r="419" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D419" s="11"/>
-      <c r="I419" s="6"/>
+      <c r="I419" s="7"/>
     </row>
     <row r="420" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D420" s="11"/>
-      <c r="I420" s="6"/>
+      <c r="I420" s="7"/>
     </row>
     <row r="421" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D421" s="11"/>
-      <c r="I421" s="6"/>
+      <c r="I421" s="7"/>
     </row>
     <row r="422" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D422" s="11"/>
-      <c r="I422" s="6"/>
+      <c r="I422" s="7"/>
     </row>
     <row r="423" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D423" s="11"/>
-      <c r="I423" s="6"/>
+      <c r="I423" s="7"/>
     </row>
     <row r="424" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D424" s="11"/>
-      <c r="I424" s="6"/>
+      <c r="I424" s="7"/>
     </row>
     <row r="425" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D425" s="11"/>
-      <c r="I425" s="6"/>
+      <c r="I425" s="7"/>
     </row>
     <row r="426" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D426" s="11"/>
-      <c r="I426" s="6"/>
+      <c r="I426" s="7"/>
     </row>
     <row r="427" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D427" s="11"/>
-      <c r="I427" s="6"/>
+      <c r="I427" s="7"/>
     </row>
     <row r="428" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D428" s="11"/>
-      <c r="I428" s="6"/>
+      <c r="I428" s="7"/>
     </row>
     <row r="429" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D429" s="11"/>
-      <c r="I429" s="6"/>
+      <c r="I429" s="7"/>
     </row>
     <row r="430" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D430" s="11"/>
-      <c r="I430" s="6"/>
+      <c r="I430" s="7"/>
     </row>
     <row r="431" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D431" s="11"/>
-      <c r="I431" s="6"/>
+      <c r="I431" s="7"/>
     </row>
     <row r="432" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D432" s="11"/>
-      <c r="I432" s="6"/>
+      <c r="I432" s="7"/>
     </row>
     <row r="433" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D433" s="11"/>
-      <c r="I433" s="6"/>
+      <c r="I433" s="7"/>
     </row>
     <row r="434" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D434" s="11"/>
-      <c r="I434" s="6"/>
+      <c r="I434" s="7"/>
     </row>
     <row r="435" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D435" s="11"/>
-      <c r="I435" s="6"/>
+      <c r="I435" s="7"/>
     </row>
     <row r="436" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D436" s="11"/>
-      <c r="I436" s="6"/>
+      <c r="I436" s="7"/>
     </row>
     <row r="437" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D437" s="11"/>
-      <c r="I437" s="6"/>
+      <c r="I437" s="7"/>
     </row>
     <row r="438" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D438" s="11"/>
-      <c r="I438" s="6"/>
+      <c r="I438" s="7"/>
     </row>
     <row r="439" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D439" s="11"/>
-      <c r="I439" s="6"/>
+      <c r="I439" s="7"/>
     </row>
     <row r="440" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D440" s="11"/>
-      <c r="I440" s="6"/>
+      <c r="I440" s="7"/>
     </row>
     <row r="441" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D441" s="11"/>
-      <c r="I441" s="6"/>
+      <c r="I441" s="7"/>
     </row>
     <row r="442" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D442" s="11"/>
-      <c r="I442" s="6"/>
+      <c r="I442" s="7"/>
     </row>
     <row r="443" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D443" s="11"/>
-      <c r="I443" s="6"/>
+      <c r="I443" s="7"/>
     </row>
     <row r="444" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D444" s="11"/>
-      <c r="I444" s="6"/>
+      <c r="I444" s="7"/>
     </row>
     <row r="445" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D445" s="11"/>
-      <c r="I445" s="6"/>
+      <c r="I445" s="7"/>
     </row>
     <row r="446" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D446" s="11"/>
-      <c r="I446" s="6"/>
+      <c r="I446" s="7"/>
     </row>
     <row r="447" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D447" s="11"/>
-      <c r="I447" s="6"/>
+      <c r="I447" s="7"/>
     </row>
     <row r="448" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D448" s="11"/>
-      <c r="I448" s="6"/>
+      <c r="I448" s="7"/>
     </row>
     <row r="449" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D449" s="11"/>
-      <c r="I449" s="6"/>
+      <c r="I449" s="7"/>
     </row>
     <row r="450" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D450" s="11"/>
-      <c r="I450" s="6"/>
+      <c r="I450" s="7"/>
     </row>
     <row r="451" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D451" s="11"/>
-      <c r="I451" s="6"/>
+      <c r="I451" s="7"/>
     </row>
     <row r="452" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D452" s="11"/>
-      <c r="I452" s="6"/>
+      <c r="I452" s="7"/>
     </row>
     <row r="453" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D453" s="11"/>
-      <c r="I453" s="6"/>
+      <c r="I453" s="7"/>
     </row>
     <row r="454" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D454" s="11"/>
-      <c r="I454" s="6"/>
+      <c r="I454" s="7"/>
     </row>
     <row r="455" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D455" s="11"/>
-      <c r="I455" s="6"/>
+      <c r="I455" s="7"/>
     </row>
     <row r="456" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D456" s="11"/>
-      <c r="I456" s="6"/>
+      <c r="I456" s="7"/>
     </row>
     <row r="457" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D457" s="11"/>
-      <c r="I457" s="6"/>
+      <c r="I457" s="7"/>
     </row>
     <row r="458" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D458" s="11"/>
-      <c r="I458" s="6"/>
+      <c r="I458" s="7"/>
     </row>
     <row r="459" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D459" s="11"/>
-      <c r="I459" s="6"/>
+      <c r="I459" s="7"/>
     </row>
     <row r="460" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D460" s="11"/>
-      <c r="I460" s="6"/>
+      <c r="I460" s="7"/>
     </row>
     <row r="461" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D461" s="11"/>
-      <c r="I461" s="6"/>
+      <c r="I461" s="7"/>
     </row>
     <row r="462" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D462" s="11"/>
-      <c r="I462" s="6"/>
+      <c r="I462" s="7"/>
     </row>
     <row r="463" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D463" s="11"/>
-      <c r="I463" s="6"/>
+      <c r="I463" s="7"/>
     </row>
     <row r="464" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D464" s="11"/>
-      <c r="I464" s="6"/>
+      <c r="I464" s="7"/>
     </row>
     <row r="465" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D465" s="11"/>
-      <c r="I465" s="6"/>
+      <c r="I465" s="7"/>
     </row>
     <row r="466" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D466" s="11"/>
-      <c r="I466" s="6"/>
+      <c r="I466" s="7"/>
     </row>
     <row r="467" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D467" s="11"/>
-      <c r="I467" s="6"/>
+      <c r="I467" s="7"/>
     </row>
     <row r="468" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D468" s="11"/>
-      <c r="I468" s="6"/>
+      <c r="I468" s="7"/>
     </row>
     <row r="469" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D469" s="11"/>
-      <c r="I469" s="6"/>
+      <c r="I469" s="7"/>
     </row>
     <row r="470" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D470" s="11"/>
-      <c r="I470" s="6"/>
+      <c r="I470" s="7"/>
     </row>
     <row r="471" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D471" s="11"/>
-      <c r="I471" s="6"/>
+      <c r="I471" s="7"/>
     </row>
     <row r="472" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D472" s="11"/>
-      <c r="I472" s="6"/>
+      <c r="I472" s="7"/>
     </row>
     <row r="473" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D473" s="11"/>
-      <c r="I473" s="6"/>
+      <c r="I473" s="7"/>
     </row>
     <row r="474" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D474" s="11"/>
-      <c r="I474" s="6"/>
+      <c r="I474" s="7"/>
     </row>
     <row r="475" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D475" s="11"/>
-      <c r="I475" s="6"/>
+      <c r="I475" s="7"/>
     </row>
     <row r="476" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D476" s="11"/>
-      <c r="I476" s="6"/>
+      <c r="I476" s="7"/>
     </row>
     <row r="477" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D477" s="11"/>
-      <c r="I477" s="6"/>
+      <c r="I477" s="7"/>
     </row>
     <row r="478" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D478" s="11"/>
-      <c r="I478" s="6"/>
+      <c r="I478" s="7"/>
     </row>
     <row r="479" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D479" s="11"/>
-      <c r="I479" s="6"/>
+      <c r="I479" s="7"/>
     </row>
     <row r="480" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D480" s="11"/>
-      <c r="I480" s="6"/>
+      <c r="I480" s="7"/>
     </row>
     <row r="481" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D481" s="11"/>
-      <c r="I481" s="6"/>
+      <c r="I481" s="7"/>
     </row>
     <row r="482" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D482" s="11"/>
-      <c r="I482" s="6"/>
+      <c r="I482" s="7"/>
     </row>
     <row r="483" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D483" s="11"/>
-      <c r="I483" s="6"/>
+      <c r="I483" s="7"/>
     </row>
     <row r="484" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D484" s="11"/>
-      <c r="I484" s="6"/>
+      <c r="I484" s="7"/>
     </row>
     <row r="485" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D485" s="11"/>
-      <c r="I485" s="6"/>
+      <c r="I485" s="7"/>
     </row>
     <row r="486" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D486" s="11"/>
-      <c r="I486" s="6"/>
+      <c r="I486" s="7"/>
     </row>
     <row r="487" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D487" s="11"/>
-      <c r="I487" s="6"/>
+      <c r="I487" s="7"/>
     </row>
     <row r="488" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D488" s="11"/>
-      <c r="I488" s="6"/>
+      <c r="I488" s="7"/>
     </row>
     <row r="489" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D489" s="11"/>
-      <c r="I489" s="6"/>
+      <c r="I489" s="7"/>
     </row>
     <row r="490" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D490" s="11"/>
-      <c r="I490" s="6"/>
+      <c r="I490" s="7"/>
     </row>
     <row r="491" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D491" s="11"/>
-      <c r="I491" s="6"/>
+      <c r="I491" s="7"/>
     </row>
     <row r="492" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D492" s="11"/>
-      <c r="I492" s="6"/>
+      <c r="I492" s="7"/>
     </row>
     <row r="493" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D493" s="11"/>
-      <c r="I493" s="6"/>
+      <c r="I493" s="7"/>
     </row>
     <row r="494" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D494" s="11"/>
-      <c r="I494" s="6"/>
+      <c r="I494" s="7"/>
     </row>
     <row r="495" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D495" s="11"/>
-      <c r="I495" s="6"/>
+      <c r="I495" s="7"/>
     </row>
     <row r="496" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D496" s="11"/>
-      <c r="I496" s="6"/>
+      <c r="I496" s="7"/>
     </row>
     <row r="497" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D497" s="11"/>
-      <c r="I497" s="6"/>
+      <c r="I497" s="7"/>
     </row>
     <row r="498" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D498" s="11"/>
-      <c r="I498" s="6"/>
+      <c r="I498" s="7"/>
     </row>
     <row r="499" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D499" s="11"/>
-      <c r="I499" s="6"/>
+      <c r="I499" s="7"/>
     </row>
     <row r="500" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D500" s="11"/>
-      <c r="I500" s="6"/>
+      <c r="I500" s="7"/>
     </row>
     <row r="501" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D501" s="11"/>
-      <c r="I501" s="6"/>
+      <c r="I501" s="7"/>
     </row>
     <row r="502" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D502" s="11"/>
-      <c r="I502" s="6"/>
+      <c r="I502" s="7"/>
     </row>
     <row r="503" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D503" s="11"/>
-      <c r="I503" s="6"/>
+      <c r="I503" s="7"/>
     </row>
     <row r="504" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D504" s="11"/>
-      <c r="I504" s="6"/>
+      <c r="I504" s="7"/>
     </row>
     <row r="505" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D505" s="11"/>
-      <c r="I505" s="6"/>
+      <c r="I505" s="7"/>
     </row>
     <row r="506" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D506" s="11"/>
-      <c r="I506" s="6"/>
+      <c r="I506" s="7"/>
     </row>
     <row r="507" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D507" s="11"/>
-      <c r="I507" s="6"/>
+      <c r="I507" s="7"/>
     </row>
     <row r="508" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D508" s="11"/>
-      <c r="I508" s="6"/>
+      <c r="I508" s="7"/>
     </row>
     <row r="509" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D509" s="11"/>
-      <c r="I509" s="6"/>
+      <c r="I509" s="7"/>
     </row>
     <row r="510" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D510" s="11"/>
-      <c r="I510" s="6"/>
+      <c r="I510" s="7"/>
     </row>
     <row r="511" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D511" s="11"/>
-      <c r="I511" s="6"/>
+      <c r="I511" s="7"/>
     </row>
     <row r="512" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D512" s="11"/>
-      <c r="I512" s="6"/>
+      <c r="I512" s="7"/>
     </row>
     <row r="513" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D513" s="11"/>
-      <c r="I513" s="6"/>
+      <c r="I513" s="7"/>
     </row>
     <row r="514" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D514" s="11"/>
-      <c r="I514" s="6"/>
+      <c r="I514" s="7"/>
     </row>
     <row r="515" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D515" s="11"/>
-      <c r="I515" s="6"/>
+      <c r="I515" s="7"/>
     </row>
     <row r="516" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D516" s="11"/>
-      <c r="I516" s="6"/>
+      <c r="I516" s="7"/>
     </row>
     <row r="517" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D517" s="11"/>
-      <c r="I517" s="6"/>
+      <c r="I517" s="7"/>
     </row>
     <row r="518" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D518" s="11"/>
-      <c r="I518" s="6"/>
+      <c r="I518" s="7"/>
     </row>
     <row r="519" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D519" s="11"/>
-      <c r="I519" s="6"/>
+      <c r="I519" s="7"/>
     </row>
     <row r="520" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D520" s="11"/>
-      <c r="I520" s="6"/>
+      <c r="I520" s="7"/>
     </row>
     <row r="521" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D521" s="11"/>
-      <c r="I521" s="6"/>
+      <c r="I521" s="7"/>
     </row>
     <row r="522" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D522" s="11"/>
-      <c r="I522" s="6"/>
+      <c r="I522" s="7"/>
     </row>
     <row r="523" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D523" s="11"/>
-      <c r="I523" s="6"/>
+      <c r="I523" s="7"/>
     </row>
     <row r="524" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D524" s="11"/>
-      <c r="I524" s="6"/>
+      <c r="I524" s="7"/>
     </row>
     <row r="525" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D525" s="11"/>
-      <c r="I525" s="6"/>
+      <c r="I525" s="7"/>
     </row>
     <row r="526" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D526" s="11"/>
-      <c r="I526" s="6"/>
+      <c r="I526" s="7"/>
     </row>
     <row r="527" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D527" s="11"/>
-      <c r="I527" s="6"/>
+      <c r="I527" s="7"/>
     </row>
     <row r="528" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D528" s="11"/>
-      <c r="I528" s="6"/>
+      <c r="I528" s="7"/>
     </row>
     <row r="529" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D529" s="11"/>
-      <c r="I529" s="6"/>
+      <c r="I529" s="7"/>
     </row>
     <row r="530" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D530" s="11"/>
-      <c r="I530" s="6"/>
+      <c r="I530" s="7"/>
     </row>
     <row r="531" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D531" s="11"/>
-      <c r="I531" s="6"/>
+      <c r="I531" s="7"/>
     </row>
     <row r="532" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D532" s="11"/>
-      <c r="I532" s="6"/>
+      <c r="I532" s="7"/>
     </row>
     <row r="533" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D533" s="11"/>
-      <c r="I533" s="6"/>
+      <c r="I533" s="7"/>
     </row>
     <row r="534" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D534" s="11"/>
-      <c r="I534" s="6"/>
+      <c r="I534" s="7"/>
     </row>
     <row r="535" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D535" s="11"/>
-      <c r="I535" s="6"/>
+      <c r="I535" s="7"/>
     </row>
     <row r="536" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D536" s="11"/>
-      <c r="I536" s="6"/>
+      <c r="I536" s="7"/>
     </row>
     <row r="537" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D537" s="11"/>
-      <c r="I537" s="6"/>
+      <c r="I537" s="7"/>
     </row>
     <row r="538" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D538" s="11"/>
-      <c r="I538" s="6"/>
+      <c r="I538" s="7"/>
     </row>
     <row r="539" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D539" s="11"/>
-      <c r="I539" s="6"/>
+      <c r="I539" s="7"/>
     </row>
     <row r="540" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D540" s="11"/>
-      <c r="I540" s="6"/>
+      <c r="I540" s="7"/>
     </row>
     <row r="541" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D541" s="11"/>
-      <c r="I541" s="6"/>
+      <c r="I541" s="7"/>
     </row>
     <row r="542" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D542" s="11"/>
-      <c r="I542" s="6"/>
+      <c r="I542" s="7"/>
     </row>
     <row r="543" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D543" s="11"/>
-      <c r="I543" s="6"/>
+      <c r="I543" s="7"/>
     </row>
     <row r="544" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D544" s="11"/>
-      <c r="I544" s="6"/>
+      <c r="I544" s="7"/>
     </row>
     <row r="545" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D545" s="11"/>
-      <c r="I545" s="6"/>
+      <c r="I545" s="7"/>
     </row>
     <row r="546" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D546" s="11"/>
-      <c r="I546" s="6"/>
+      <c r="I546" s="7"/>
     </row>
     <row r="547" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D547" s="11"/>
-      <c r="I547" s="6"/>
+      <c r="I547" s="7"/>
     </row>
     <row r="548" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D548" s="11"/>
-      <c r="I548" s="6"/>
+      <c r="I548" s="7"/>
     </row>
     <row r="549" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D549" s="11"/>
-      <c r="I549" s="6"/>
+      <c r="I549" s="7"/>
     </row>
     <row r="550" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D550" s="11"/>
-      <c r="I550" s="6"/>
+      <c r="I550" s="7"/>
     </row>
     <row r="551" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D551" s="11"/>
-      <c r="I551" s="6"/>
+      <c r="I551" s="7"/>
     </row>
     <row r="552" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D552" s="11"/>
-      <c r="I552" s="6"/>
+      <c r="I552" s="7"/>
     </row>
     <row r="553" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D553" s="11"/>
-      <c r="I553" s="6"/>
+      <c r="I553" s="7"/>
     </row>
     <row r="554" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D554" s="11"/>
-      <c r="I554" s="6"/>
+      <c r="I554" s="7"/>
     </row>
     <row r="555" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D555" s="11"/>
-      <c r="I555" s="6"/>
+      <c r="I555" s="7"/>
     </row>
     <row r="556" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D556" s="11"/>
-      <c r="I556" s="6"/>
+      <c r="I556" s="7"/>
     </row>
     <row r="557" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D557" s="11"/>
-      <c r="I557" s="6"/>
+      <c r="I557" s="7"/>
     </row>
     <row r="558" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D558" s="11"/>
-      <c r="I558" s="6"/>
+      <c r="I558" s="7"/>
     </row>
     <row r="559" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D559" s="11"/>
-      <c r="I559" s="6"/>
+      <c r="I559" s="7"/>
     </row>
     <row r="560" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D560" s="11"/>
-      <c r="I560" s="6"/>
+      <c r="I560" s="7"/>
     </row>
     <row r="561" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D561" s="11"/>
-      <c r="I561" s="6"/>
+      <c r="I561" s="7"/>
     </row>
     <row r="562" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D562" s="11"/>
-      <c r="I562" s="6"/>
+      <c r="I562" s="7"/>
     </row>
     <row r="563" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D563" s="11"/>
-      <c r="I563" s="6"/>
+      <c r="I563" s="7"/>
     </row>
     <row r="564" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D564" s="11"/>
-      <c r="I564" s="6"/>
+      <c r="I564" s="7"/>
     </row>
     <row r="565" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D565" s="11"/>
-      <c r="I565" s="6"/>
+      <c r="I565" s="7"/>
     </row>
     <row r="566" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D566" s="11"/>
-      <c r="I566" s="6"/>
+      <c r="I566" s="7"/>
     </row>
     <row r="567" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D567" s="11"/>
-      <c r="I567" s="6"/>
+      <c r="I567" s="7"/>
     </row>
     <row r="568" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D568" s="11"/>
-      <c r="I568" s="6"/>
+      <c r="I568" s="7"/>
     </row>
     <row r="569" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D569" s="11"/>
-      <c r="I569" s="6"/>
+      <c r="I569" s="7"/>
     </row>
     <row r="570" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D570" s="11"/>
-      <c r="I570" s="6"/>
+      <c r="I570" s="7"/>
     </row>
     <row r="571" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D571" s="11"/>
-      <c r="I571" s="6"/>
+      <c r="I571" s="7"/>
     </row>
     <row r="572" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D572" s="11"/>
-      <c r="I572" s="6"/>
+      <c r="I572" s="7"/>
     </row>
     <row r="573" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D573" s="11"/>
-      <c r="I573" s="6"/>
+      <c r="I573" s="7"/>
     </row>
     <row r="574" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D574" s="11"/>
-      <c r="I574" s="6"/>
+      <c r="I574" s="7"/>
     </row>
     <row r="575" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D575" s="11"/>
-      <c r="I575" s="6"/>
+      <c r="I575" s="7"/>
     </row>
     <row r="576" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D576" s="11"/>
-      <c r="I576" s="6"/>
+      <c r="I576" s="7"/>
     </row>
     <row r="577" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D577" s="11"/>
-      <c r="I577" s="6"/>
+      <c r="I577" s="7"/>
     </row>
     <row r="578" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D578" s="11"/>
-      <c r="I578" s="6"/>
+      <c r="I578" s="7"/>
     </row>
     <row r="579" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D579" s="11"/>
-      <c r="I579" s="6"/>
+      <c r="I579" s="7"/>
     </row>
     <row r="580" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D580" s="11"/>
-      <c r="I580" s="6"/>
+      <c r="I580" s="7"/>
     </row>
     <row r="581" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D581" s="11"/>
-      <c r="I581" s="6"/>
+      <c r="I581" s="7"/>
     </row>
     <row r="582" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D582" s="11"/>
-      <c r="I582" s="6"/>
+      <c r="I582" s="7"/>
     </row>
     <row r="583" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D583" s="11"/>
-      <c r="I583" s="6"/>
+      <c r="I583" s="7"/>
     </row>
     <row r="584" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D584" s="11"/>
-      <c r="I584" s="6"/>
+      <c r="I584" s="7"/>
     </row>
     <row r="585" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D585" s="11"/>
-      <c r="I585" s="6"/>
+      <c r="I585" s="7"/>
     </row>
     <row r="586" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D586" s="11"/>
-      <c r="I586" s="6"/>
+      <c r="I586" s="7"/>
     </row>
     <row r="587" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D587" s="11"/>
-      <c r="I587" s="6"/>
+      <c r="I587" s="7"/>
     </row>
     <row r="588" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D588" s="11"/>
-      <c r="I588" s="6"/>
+      <c r="I588" s="7"/>
     </row>
     <row r="589" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D589" s="11"/>
-      <c r="I589" s="6"/>
+      <c r="I589" s="7"/>
     </row>
     <row r="590" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D590" s="11"/>
-      <c r="I590" s="6"/>
+      <c r="I590" s="7"/>
     </row>
     <row r="591" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D591" s="11"/>
-      <c r="I591" s="6"/>
+      <c r="I591" s="7"/>
     </row>
     <row r="592" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D592" s="11"/>
-      <c r="I592" s="6"/>
+      <c r="I592" s="7"/>
     </row>
     <row r="593" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D593" s="11"/>
-      <c r="I593" s="6"/>
+      <c r="I593" s="7"/>
     </row>
     <row r="594" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D594" s="11"/>
-      <c r="I594" s="6"/>
+      <c r="I594" s="7"/>
     </row>
     <row r="595" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D595" s="11"/>
-      <c r="I595" s="6"/>
+      <c r="I595" s="7"/>
     </row>
     <row r="596" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D596" s="11"/>
-      <c r="I596" s="6"/>
+      <c r="I596" s="7"/>
     </row>
     <row r="597" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D597" s="11"/>
-      <c r="I597" s="6"/>
+      <c r="I597" s="7"/>
     </row>
     <row r="598" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D598" s="11"/>
-      <c r="I598" s="6"/>
+      <c r="I598" s="7"/>
     </row>
     <row r="599" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D599" s="11"/>
-      <c r="I599" s="6"/>
+      <c r="I599" s="7"/>
     </row>
     <row r="600" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D600" s="11"/>
-      <c r="I600" s="6"/>
+      <c r="I600" s="7"/>
     </row>
     <row r="601" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D601" s="11"/>
-      <c r="I601" s="6"/>
+      <c r="I601" s="7"/>
     </row>
     <row r="602" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D602" s="11"/>
-      <c r="I602" s="6"/>
+      <c r="I602" s="7"/>
     </row>
     <row r="603" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D603" s="11"/>
-      <c r="I603" s="6"/>
+      <c r="I603" s="7"/>
     </row>
     <row r="604" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D604" s="11"/>
-      <c r="I604" s="6"/>
+      <c r="I604" s="7"/>
     </row>
     <row r="605" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D605" s="11"/>
-      <c r="I605" s="6"/>
+      <c r="I605" s="7"/>
     </row>
     <row r="606" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D606" s="11"/>
-      <c r="I606" s="6"/>
+      <c r="I606" s="7"/>
     </row>
     <row r="607" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D607" s="11"/>
-      <c r="I607" s="6"/>
+      <c r="I607" s="7"/>
     </row>
     <row r="608" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D608" s="11"/>
-      <c r="I608" s="6"/>
+      <c r="I608" s="7"/>
     </row>
     <row r="609" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D609" s="11"/>
-      <c r="I609" s="6"/>
+      <c r="I609" s="7"/>
     </row>
     <row r="610" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D610" s="11"/>
-      <c r="I610" s="6"/>
+      <c r="I610" s="7"/>
     </row>
     <row r="611" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D611" s="11"/>
-      <c r="I611" s="6"/>
+      <c r="I611" s="7"/>
     </row>
     <row r="612" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D612" s="11"/>
-      <c r="I612" s="6"/>
+      <c r="I612" s="7"/>
     </row>
     <row r="613" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D613" s="11"/>
-      <c r="I613" s="6"/>
+      <c r="I613" s="7"/>
     </row>
     <row r="614" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D614" s="11"/>
-      <c r="I614" s="6"/>
+      <c r="I614" s="7"/>
     </row>
     <row r="615" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D615" s="11"/>
-      <c r="I615" s="6"/>
+      <c r="I615" s="7"/>
     </row>
     <row r="616" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D616" s="11"/>
-      <c r="I616" s="6"/>
+      <c r="I616" s="7"/>
     </row>
     <row r="617" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D617" s="11"/>
-      <c r="I617" s="6"/>
+      <c r="I617" s="7"/>
     </row>
     <row r="618" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D618" s="11"/>
-      <c r="I618" s="6"/>
+      <c r="I618" s="7"/>
     </row>
     <row r="619" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D619" s="11"/>
-      <c r="I619" s="6"/>
+      <c r="I619" s="7"/>
     </row>
     <row r="620" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D620" s="11"/>
-      <c r="I620" s="6"/>
+      <c r="I620" s="7"/>
     </row>
     <row r="621" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D621" s="11"/>
-      <c r="I621" s="6"/>
+      <c r="I621" s="7"/>
     </row>
     <row r="622" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D622" s="11"/>
-      <c r="I622" s="6"/>
+      <c r="I622" s="7"/>
     </row>
     <row r="623" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D623" s="11"/>
-      <c r="I623" s="6"/>
+      <c r="I623" s="7"/>
     </row>
     <row r="624" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D624" s="11"/>
-      <c r="I624" s="6"/>
+      <c r="I624" s="7"/>
     </row>
     <row r="625" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D625" s="11"/>
-      <c r="I625" s="6"/>
+      <c r="I625" s="7"/>
     </row>
     <row r="626" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D626" s="11"/>
-      <c r="I626" s="6"/>
+      <c r="I626" s="7"/>
     </row>
     <row r="627" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D627" s="11"/>
-      <c r="I627" s="6"/>
+      <c r="I627" s="7"/>
     </row>
     <row r="628" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D628" s="11"/>
-      <c r="I628" s="6"/>
+      <c r="I628" s="7"/>
     </row>
     <row r="629" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D629" s="11"/>
-      <c r="I629" s="6"/>
+      <c r="I629" s="7"/>
     </row>
     <row r="630" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D630" s="11"/>
-      <c r="I630" s="6"/>
+      <c r="I630" s="7"/>
     </row>
     <row r="631" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D631" s="11"/>
-      <c r="I631" s="6"/>
+      <c r="I631" s="7"/>
     </row>
     <row r="632" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D632" s="11"/>
-      <c r="I632" s="6"/>
+      <c r="I632" s="7"/>
     </row>
     <row r="633" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D633" s="11"/>
-      <c r="I633" s="6"/>
+      <c r="I633" s="7"/>
     </row>
     <row r="634" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D634" s="11"/>
-      <c r="I634" s="6"/>
+      <c r="I634" s="7"/>
     </row>
     <row r="635" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D635" s="11"/>
-      <c r="I635" s="6"/>
+      <c r="I635" s="7"/>
     </row>
     <row r="636" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D636" s="11"/>
-      <c r="I636" s="6"/>
+      <c r="I636" s="7"/>
     </row>
     <row r="637" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D637" s="11"/>
-      <c r="I637" s="6"/>
+      <c r="I637" s="7"/>
     </row>
     <row r="638" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D638" s="11"/>
-      <c r="I638" s="6"/>
+      <c r="I638" s="7"/>
     </row>
     <row r="639" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D639" s="11"/>
-      <c r="I639" s="6"/>
+      <c r="I639" s="7"/>
     </row>
     <row r="640" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D640" s="11"/>
-      <c r="I640" s="6"/>
+      <c r="I640" s="7"/>
     </row>
     <row r="641" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D641" s="11"/>
-      <c r="I641" s="6"/>
+      <c r="I641" s="7"/>
     </row>
     <row r="642" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D642" s="11"/>
-      <c r="I642" s="6"/>
+      <c r="I642" s="7"/>
     </row>
     <row r="643" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D643" s="11"/>
-      <c r="I643" s="6"/>
+      <c r="I643" s="7"/>
     </row>
     <row r="644" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D644" s="11"/>
-      <c r="I644" s="6"/>
+      <c r="I644" s="7"/>
     </row>
     <row r="645" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D645" s="11"/>
-      <c r="I645" s="6"/>
+      <c r="I645" s="7"/>
     </row>
     <row r="646" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D646" s="11"/>
-      <c r="I646" s="6"/>
+      <c r="I646" s="7"/>
     </row>
     <row r="647" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D647" s="11"/>
-      <c r="I647" s="6"/>
+      <c r="I647" s="7"/>
     </row>
     <row r="648" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D648" s="11"/>
-      <c r="I648" s="6"/>
+      <c r="I648" s="7"/>
     </row>
     <row r="649" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D649" s="11"/>
-      <c r="I649" s="6"/>
+      <c r="I649" s="7"/>
     </row>
     <row r="650" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D650" s="11"/>
-      <c r="I650" s="6"/>
+      <c r="I650" s="7"/>
     </row>
     <row r="651" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D651" s="11"/>
-      <c r="I651" s="6"/>
+      <c r="I651" s="7"/>
     </row>
     <row r="652" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D652" s="11"/>
-      <c r="I652" s="6"/>
+      <c r="I652" s="7"/>
     </row>
     <row r="653" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D653" s="11"/>
-      <c r="I653" s="6"/>
+      <c r="I653" s="7"/>
     </row>
     <row r="654" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D654" s="11"/>
-      <c r="I654" s="6"/>
+      <c r="I654" s="7"/>
     </row>
     <row r="655" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D655" s="11"/>
-      <c r="I655" s="6"/>
+      <c r="I655" s="7"/>
     </row>
     <row r="656" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D656" s="11"/>
-      <c r="I656" s="6"/>
+      <c r="I656" s="7"/>
     </row>
     <row r="657" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D657" s="11"/>
-      <c r="I657" s="6"/>
+      <c r="I657" s="7"/>
     </row>
     <row r="658" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D658" s="11"/>
-      <c r="I658" s="6"/>
+      <c r="I658" s="7"/>
     </row>
     <row r="659" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D659" s="11"/>
-      <c r="I659" s="6"/>
+      <c r="I659" s="7"/>
     </row>
     <row r="660" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D660" s="11"/>
-      <c r="I660" s="6"/>
+      <c r="I660" s="7"/>
     </row>
     <row r="661" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D661" s="11"/>
-      <c r="I661" s="6"/>
+      <c r="I661" s="7"/>
     </row>
     <row r="662" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D662" s="11"/>
-      <c r="I662" s="6"/>
+      <c r="I662" s="7"/>
     </row>
     <row r="663" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D663" s="11"/>
-      <c r="I663" s="6"/>
+      <c r="I663" s="7"/>
     </row>
     <row r="664" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D664" s="11"/>
-      <c r="I664" s="6"/>
+      <c r="I664" s="7"/>
     </row>
     <row r="665" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D665" s="11"/>
-      <c r="I665" s="6"/>
+      <c r="I665" s="7"/>
     </row>
     <row r="666" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D666" s="11"/>
-      <c r="I666" s="6"/>
+      <c r="I666" s="7"/>
     </row>
     <row r="667" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D667" s="11"/>
-      <c r="I667" s="6"/>
+      <c r="I667" s="7"/>
     </row>
     <row r="668" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D668" s="11"/>
-      <c r="I668" s="6"/>
+      <c r="I668" s="7"/>
     </row>
     <row r="669" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D669" s="11"/>
-      <c r="I669" s="6"/>
+      <c r="I669" s="7"/>
     </row>
     <row r="670" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D670" s="11"/>
-      <c r="I670" s="6"/>
+      <c r="I670" s="7"/>
     </row>
     <row r="671" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D671" s="11"/>
-      <c r="I671" s="6"/>
+      <c r="I671" s="7"/>
     </row>
     <row r="672" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D672" s="11"/>
-      <c r="I672" s="6"/>
+      <c r="I672" s="7"/>
     </row>
     <row r="673" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D673" s="11"/>
-      <c r="I673" s="6"/>
+      <c r="I673" s="7"/>
     </row>
     <row r="674" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D674" s="11"/>
-      <c r="I674" s="6"/>
+      <c r="I674" s="7"/>
     </row>
     <row r="675" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D675" s="11"/>
-      <c r="I675" s="6"/>
+      <c r="I675" s="7"/>
     </row>
     <row r="676" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D676" s="11"/>
-      <c r="I676" s="6"/>
+      <c r="I676" s="7"/>
     </row>
     <row r="677" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D677" s="11"/>
-      <c r="I677" s="6"/>
+      <c r="I677" s="7"/>
     </row>
     <row r="678" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D678" s="11"/>
-      <c r="I678" s="6"/>
+      <c r="I678" s="7"/>
     </row>
     <row r="679" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D679" s="11"/>
-      <c r="I679" s="6"/>
+      <c r="I679" s="7"/>
     </row>
     <row r="680" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D680" s="11"/>
-      <c r="I680" s="6"/>
+      <c r="I680" s="7"/>
     </row>
     <row r="681" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D681" s="11"/>
-      <c r="I681" s="6"/>
+      <c r="I681" s="7"/>
     </row>
     <row r="682" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D682" s="11"/>
-      <c r="I682" s="6"/>
+      <c r="I682" s="7"/>
     </row>
     <row r="683" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D683" s="11"/>
-      <c r="I683" s="6"/>
+      <c r="I683" s="7"/>
     </row>
     <row r="684" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D684" s="11"/>
-      <c r="I684" s="6"/>
+      <c r="I684" s="7"/>
     </row>
     <row r="685" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D685" s="11"/>
-      <c r="I685" s="6"/>
+      <c r="I685" s="7"/>
     </row>
     <row r="686" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D686" s="11"/>
-      <c r="I686" s="6"/>
+      <c r="I686" s="7"/>
     </row>
     <row r="687" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D687" s="11"/>
-      <c r="I687" s="6"/>
+      <c r="I687" s="7"/>
     </row>
     <row r="688" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D688" s="11"/>
-      <c r="I688" s="6"/>
+      <c r="I688" s="7"/>
     </row>
     <row r="689" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D689" s="11"/>
-      <c r="I689" s="6"/>
+      <c r="I689" s="7"/>
     </row>
     <row r="690" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D690" s="11"/>
-      <c r="I690" s="6"/>
+      <c r="I690" s="7"/>
     </row>
     <row r="691" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D691" s="11"/>
-      <c r="I691" s="6"/>
+      <c r="I691" s="7"/>
     </row>
     <row r="692" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D692" s="11"/>
-      <c r="I692" s="6"/>
+      <c r="I692" s="7"/>
     </row>
     <row r="693" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D693" s="11"/>
-      <c r="I693" s="6"/>
+      <c r="I693" s="7"/>
     </row>
     <row r="694" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D694" s="11"/>
-      <c r="I694" s="6"/>
+      <c r="I694" s="7"/>
     </row>
     <row r="695" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D695" s="11"/>
-      <c r="I695" s="6"/>
+      <c r="I695" s="7"/>
     </row>
     <row r="696" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D696" s="11"/>
-      <c r="I696" s="6"/>
+      <c r="I696" s="7"/>
     </row>
     <row r="697" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D697" s="11"/>
-      <c r="I697" s="6"/>
+      <c r="I697" s="7"/>
     </row>
     <row r="698" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D698" s="11"/>
-      <c r="I698" s="6"/>
+      <c r="I698" s="7"/>
     </row>
     <row r="699" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D699" s="11"/>
-      <c r="I699" s="6"/>
+      <c r="I699" s="7"/>
     </row>
     <row r="700" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D700" s="11"/>
-      <c r="I700" s="6"/>
+      <c r="I700" s="7"/>
     </row>
     <row r="701" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D701" s="11"/>
-      <c r="I701" s="6"/>
+      <c r="I701" s="7"/>
     </row>
     <row r="702" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D702" s="11"/>
-      <c r="I702" s="6"/>
+      <c r="I702" s="7"/>
     </row>
     <row r="703" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D703" s="11"/>
-      <c r="I703" s="6"/>
+      <c r="I703" s="7"/>
     </row>
     <row r="704" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D704" s="11"/>
-      <c r="I704" s="6"/>
+      <c r="I704" s="7"/>
     </row>
     <row r="705" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D705" s="11"/>
-      <c r="I705" s="6"/>
+      <c r="I705" s="7"/>
     </row>
     <row r="706" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D706" s="11"/>
-      <c r="I706" s="6"/>
+      <c r="I706" s="7"/>
     </row>
     <row r="707" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D707" s="11"/>
-      <c r="I707" s="6"/>
+      <c r="I707" s="7"/>
     </row>
     <row r="708" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D708" s="11"/>
-      <c r="I708" s="6"/>
+      <c r="I708" s="7"/>
     </row>
     <row r="709" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D709" s="11"/>
-      <c r="I709" s="6"/>
+      <c r="I709" s="7"/>
     </row>
     <row r="710" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D710" s="11"/>
-      <c r="I710" s="6"/>
+      <c r="I710" s="7"/>
     </row>
     <row r="711" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D711" s="11"/>
-      <c r="I711" s="6"/>
+      <c r="I711" s="7"/>
     </row>
     <row r="712" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D712" s="11"/>
-      <c r="I712" s="6"/>
+      <c r="I712" s="7"/>
     </row>
     <row r="713" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D713" s="11"/>
-      <c r="I713" s="6"/>
+      <c r="I713" s="7"/>
     </row>
     <row r="714" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D714" s="11"/>
-      <c r="I714" s="6"/>
+      <c r="I714" s="7"/>
     </row>
     <row r="715" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D715" s="11"/>
-      <c r="I715" s="6"/>
+      <c r="I715" s="7"/>
     </row>
     <row r="716" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D716" s="11"/>
-      <c r="I716" s="6"/>
+      <c r="I716" s="7"/>
     </row>
     <row r="717" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D717" s="11"/>
-      <c r="I717" s="6"/>
+      <c r="I717" s="7"/>
     </row>
     <row r="718" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D718" s="11"/>
-      <c r="I718" s="6"/>
+      <c r="I718" s="7"/>
     </row>
     <row r="719" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D719" s="11"/>
-      <c r="I719" s="6"/>
+      <c r="I719" s="7"/>
     </row>
     <row r="720" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D720" s="11"/>
-      <c r="I720" s="6"/>
+      <c r="I720" s="7"/>
     </row>
     <row r="721" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D721" s="11"/>
-      <c r="I721" s="6"/>
+      <c r="I721" s="7"/>
     </row>
     <row r="722" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D722" s="11"/>
-      <c r="I722" s="6"/>
+      <c r="I722" s="7"/>
     </row>
     <row r="723" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D723" s="11"/>
-      <c r="I723" s="6"/>
+      <c r="I723" s="7"/>
     </row>
     <row r="724" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D724" s="11"/>
-      <c r="I724" s="6"/>
+      <c r="I724" s="7"/>
     </row>
     <row r="725" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D725" s="11"/>
-      <c r="I725" s="6"/>
+      <c r="I725" s="7"/>
     </row>
     <row r="726" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D726" s="11"/>
-      <c r="I726" s="6"/>
+      <c r="I726" s="7"/>
     </row>
     <row r="727" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D727" s="11"/>
-      <c r="I727" s="6"/>
+      <c r="I727" s="7"/>
     </row>
     <row r="728" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D728" s="11"/>
-      <c r="I728" s="6"/>
+      <c r="I728" s="7"/>
     </row>
     <row r="729" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D729" s="11"/>
-      <c r="I729" s="6"/>
+      <c r="I729" s="7"/>
     </row>
     <row r="730" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D730" s="11"/>
-      <c r="I730" s="6"/>
+      <c r="I730" s="7"/>
     </row>
     <row r="731" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D731" s="11"/>
-      <c r="I731" s="6"/>
+      <c r="I731" s="7"/>
     </row>
     <row r="732" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D732" s="11"/>
-      <c r="I732" s="6"/>
+      <c r="I732" s="7"/>
     </row>
     <row r="733" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D733" s="11"/>
-      <c r="I733" s="6"/>
+      <c r="I733" s="7"/>
     </row>
     <row r="734" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D734" s="11"/>
-      <c r="I734" s="6"/>
+      <c r="I734" s="7"/>
     </row>
     <row r="735" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D735" s="11"/>
-      <c r="I735" s="6"/>
+      <c r="I735" s="7"/>
     </row>
     <row r="736" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D736" s="11"/>
-      <c r="I736" s="6"/>
+      <c r="I736" s="7"/>
     </row>
     <row r="737" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D737" s="11"/>
-      <c r="I737" s="6"/>
+      <c r="I737" s="7"/>
     </row>
     <row r="738" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D738" s="11"/>
-      <c r="I738" s="6"/>
+      <c r="I738" s="7"/>
     </row>
     <row r="739" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D739" s="11"/>
-      <c r="I739" s="6"/>
+      <c r="I739" s="7"/>
     </row>
     <row r="740" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D740" s="11"/>
-      <c r="I740" s="6"/>
+      <c r="I740" s="7"/>
     </row>
     <row r="741" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D741" s="11"/>
-      <c r="I741" s="6"/>
+      <c r="I741" s="7"/>
     </row>
     <row r="742" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D742" s="11"/>
-      <c r="I742" s="6"/>
+      <c r="I742" s="7"/>
     </row>
     <row r="743" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D743" s="11"/>
-      <c r="I743" s="6"/>
+      <c r="I743" s="7"/>
     </row>
     <row r="744" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D744" s="11"/>
-      <c r="I744" s="6"/>
+      <c r="I744" s="7"/>
     </row>
     <row r="745" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D745" s="11"/>
-      <c r="I745" s="6"/>
+      <c r="I745" s="7"/>
     </row>
     <row r="746" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D746" s="11"/>
-      <c r="I746" s="6"/>
+      <c r="I746" s="7"/>
     </row>
     <row r="747" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D747" s="11"/>
-      <c r="I747" s="6"/>
+      <c r="I747" s="7"/>
     </row>
     <row r="748" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D748" s="11"/>
-      <c r="I748" s="6"/>
+      <c r="I748" s="7"/>
     </row>
     <row r="749" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D749" s="11"/>
-      <c r="I749" s="6"/>
+      <c r="I749" s="7"/>
     </row>
     <row r="750" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D750" s="11"/>
-      <c r="I750" s="6"/>
+      <c r="I750" s="7"/>
     </row>
     <row r="751" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D751" s="11"/>
-      <c r="I751" s="6"/>
+      <c r="I751" s="7"/>
     </row>
     <row r="752" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D752" s="11"/>
-      <c r="I752" s="6"/>
+      <c r="I752" s="7"/>
     </row>
     <row r="753" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D753" s="11"/>
-      <c r="I753" s="6"/>
+      <c r="I753" s="7"/>
     </row>
     <row r="754" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D754" s="11"/>
-      <c r="I754" s="6"/>
+      <c r="I754" s="7"/>
     </row>
     <row r="755" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D755" s="11"/>
-      <c r="I755" s="6"/>
+      <c r="I755" s="7"/>
     </row>
     <row r="756" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D756" s="11"/>
-      <c r="I756" s="6"/>
+      <c r="I756" s="7"/>
     </row>
     <row r="757" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D757" s="11"/>
-      <c r="I757" s="6"/>
+      <c r="I757" s="7"/>
     </row>
     <row r="758" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D758" s="11"/>
-      <c r="I758" s="6"/>
+      <c r="I758" s="7"/>
     </row>
     <row r="759" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D759" s="11"/>
-      <c r="I759" s="6"/>
+      <c r="I759" s="7"/>
     </row>
     <row r="760" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D760" s="11"/>
-      <c r="I760" s="6"/>
+      <c r="I760" s="7"/>
     </row>
     <row r="761" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D761" s="11"/>
-      <c r="I761" s="6"/>
+      <c r="I761" s="7"/>
     </row>
     <row r="762" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D762" s="11"/>
-      <c r="I762" s="6"/>
+      <c r="I762" s="7"/>
     </row>
     <row r="763" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D763" s="11"/>
-      <c r="I763" s="6"/>
+      <c r="I763" s="7"/>
     </row>
     <row r="764" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D764" s="11"/>
-      <c r="I764" s="6"/>
+      <c r="I764" s="7"/>
     </row>
     <row r="765" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D765" s="11"/>
-      <c r="I765" s="6"/>
+      <c r="I765" s="7"/>
     </row>
     <row r="766" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D766" s="11"/>
-      <c r="I766" s="6"/>
+      <c r="I766" s="7"/>
     </row>
     <row r="767" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D767" s="11"/>
-      <c r="I767" s="6"/>
+      <c r="I767" s="7"/>
     </row>
     <row r="768" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D768" s="11"/>
-      <c r="I768" s="6"/>
+      <c r="I768" s="7"/>
     </row>
     <row r="769" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D769" s="11"/>
-      <c r="I769" s="6"/>
+      <c r="I769" s="7"/>
     </row>
     <row r="770" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D770" s="11"/>
-      <c r="I770" s="6"/>
+      <c r="I770" s="7"/>
     </row>
     <row r="771" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D771" s="11"/>
-      <c r="I771" s="6"/>
+      <c r="I771" s="7"/>
     </row>
     <row r="772" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D772" s="11"/>
-      <c r="I772" s="6"/>
+      <c r="I772" s="7"/>
     </row>
     <row r="773" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D773" s="11"/>
-      <c r="I773" s="6"/>
+      <c r="I773" s="7"/>
     </row>
     <row r="774" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D774" s="11"/>
-      <c r="I774" s="6"/>
+      <c r="I774" s="7"/>
     </row>
     <row r="775" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D775" s="11"/>
-      <c r="I775" s="6"/>
+      <c r="I775" s="7"/>
     </row>
     <row r="776" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D776" s="11"/>
-      <c r="I776" s="6"/>
+      <c r="I776" s="7"/>
     </row>
     <row r="777" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D777" s="11"/>
-      <c r="I777" s="6"/>
+      <c r="I777" s="7"/>
     </row>
     <row r="778" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D778" s="11"/>
-      <c r="I778" s="6"/>
+      <c r="I778" s="7"/>
     </row>
     <row r="779" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D779" s="11"/>
-      <c r="I779" s="6"/>
+      <c r="I779" s="7"/>
     </row>
     <row r="780" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D780" s="11"/>
-      <c r="I780" s="6"/>
+      <c r="I780" s="7"/>
     </row>
     <row r="781" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D781" s="11"/>
-      <c r="I781" s="6"/>
+      <c r="I781" s="7"/>
     </row>
     <row r="782" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D782" s="11"/>
-      <c r="I782" s="6"/>
+      <c r="I782" s="7"/>
     </row>
     <row r="783" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D783" s="11"/>
-      <c r="I783" s="6"/>
+      <c r="I783" s="7"/>
     </row>
     <row r="784" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D784" s="11"/>
-      <c r="I784" s="6"/>
+      <c r="I784" s="7"/>
     </row>
     <row r="785" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D785" s="11"/>
-      <c r="I785" s="6"/>
+      <c r="I785" s="7"/>
     </row>
     <row r="786" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D786" s="11"/>
-      <c r="I786" s="6"/>
+      <c r="I786" s="7"/>
     </row>
     <row r="787" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D787" s="11"/>
-      <c r="I787" s="6"/>
+      <c r="I787" s="7"/>
     </row>
     <row r="788" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D788" s="11"/>
-      <c r="I788" s="6"/>
+      <c r="I788" s="7"/>
     </row>
     <row r="789" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D789" s="11"/>
-      <c r="I789" s="6"/>
+      <c r="I789" s="7"/>
     </row>
     <row r="790" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D790" s="11"/>
-      <c r="I790" s="6"/>
+      <c r="I790" s="7"/>
     </row>
     <row r="791" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D791" s="11"/>
-      <c r="I791" s="6"/>
+      <c r="I791" s="7"/>
     </row>
     <row r="792" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D792" s="11"/>
-      <c r="I792" s="6"/>
+      <c r="I792" s="7"/>
     </row>
     <row r="793" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D793" s="11"/>
-      <c r="I793" s="6"/>
+      <c r="I793" s="7"/>
     </row>
     <row r="794" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D794" s="11"/>
-      <c r="I794" s="6"/>
+      <c r="I794" s="7"/>
     </row>
     <row r="795" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D795" s="11"/>
-      <c r="I795" s="6"/>
+      <c r="I795" s="7"/>
     </row>
     <row r="796" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D796" s="11"/>
-      <c r="I796" s="6"/>
+      <c r="I796" s="7"/>
     </row>
     <row r="797" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D797" s="11"/>
-      <c r="I797" s="6"/>
+      <c r="I797" s="7"/>
     </row>
     <row r="798" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D798" s="11"/>
-      <c r="I798" s="6"/>
+      <c r="I798" s="7"/>
     </row>
     <row r="799" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D799" s="11"/>
-      <c r="I799" s="6"/>
+      <c r="I799" s="7"/>
     </row>
     <row r="800" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D800" s="11"/>
-      <c r="I800" s="6"/>
+      <c r="I800" s="7"/>
     </row>
     <row r="801" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D801" s="11"/>
-      <c r="I801" s="6"/>
+      <c r="I801" s="7"/>
     </row>
     <row r="802" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D802" s="11"/>
-      <c r="I802" s="6"/>
+      <c r="I802" s="7"/>
     </row>
     <row r="803" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D803" s="11"/>
-      <c r="I803" s="6"/>
+      <c r="I803" s="7"/>
     </row>
     <row r="804" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D804" s="11"/>
-      <c r="I804" s="6"/>
+      <c r="I804" s="7"/>
     </row>
     <row r="805" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D805" s="11"/>
-      <c r="I805" s="6"/>
+      <c r="I805" s="7"/>
     </row>
     <row r="806" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D806" s="11"/>
-      <c r="I806" s="6"/>
+      <c r="I806" s="7"/>
     </row>
     <row r="807" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D807" s="11"/>
-      <c r="I807" s="6"/>
+      <c r="I807" s="7"/>
     </row>
     <row r="808" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D808" s="11"/>
-      <c r="I808" s="6"/>
+      <c r="I808" s="7"/>
     </row>
     <row r="809" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D809" s="11"/>
-      <c r="I809" s="6"/>
+      <c r="I809" s="7"/>
     </row>
     <row r="810" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D810" s="11"/>
-      <c r="I810" s="6"/>
+      <c r="I810" s="7"/>
     </row>
     <row r="811" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D811" s="11"/>
-      <c r="I811" s="6"/>
+      <c r="I811" s="7"/>
     </row>
     <row r="812" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D812" s="11"/>
-      <c r="I812" s="6"/>
+      <c r="I812" s="7"/>
     </row>
     <row r="813" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D813" s="11"/>
-      <c r="I813" s="6"/>
+      <c r="I813" s="7"/>
     </row>
     <row r="814" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D814" s="11"/>
-      <c r="I814" s="6"/>
+      <c r="I814" s="7"/>
     </row>
     <row r="815" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D815" s="11"/>
-      <c r="I815" s="6"/>
+      <c r="I815" s="7"/>
     </row>
     <row r="816" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D816" s="11"/>
-      <c r="I816" s="6"/>
+      <c r="I816" s="7"/>
     </row>
     <row r="817" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D817" s="11"/>
-      <c r="I817" s="6"/>
+      <c r="I817" s="7"/>
     </row>
     <row r="818" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D818" s="11"/>
-      <c r="I818" s="6"/>
+      <c r="I818" s="7"/>
     </row>
     <row r="819" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D819" s="11"/>
-      <c r="I819" s="6"/>
+      <c r="I819" s="7"/>
     </row>
     <row r="820" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D820" s="11"/>
-      <c r="I820" s="6"/>
+      <c r="I820" s="7"/>
     </row>
     <row r="821" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D821" s="11"/>
-      <c r="I821" s="6"/>
+      <c r="I821" s="7"/>
     </row>
     <row r="822" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D822" s="11"/>
-      <c r="I822" s="6"/>
+      <c r="I822" s="7"/>
     </row>
     <row r="823" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D823" s="11"/>
-      <c r="I823" s="6"/>
+      <c r="I823" s="7"/>
     </row>
     <row r="824" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D824" s="11"/>
-      <c r="I824" s="6"/>
+      <c r="I824" s="7"/>
     </row>
     <row r="825" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D825" s="11"/>
-      <c r="I825" s="6"/>
+      <c r="I825" s="7"/>
     </row>
     <row r="826" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D826" s="11"/>
-      <c r="I826" s="6"/>
+      <c r="I826" s="7"/>
     </row>
     <row r="827" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D827" s="11"/>
-      <c r="I827" s="6"/>
+      <c r="I827" s="7"/>
     </row>
     <row r="828" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D828" s="11"/>
-      <c r="I828" s="6"/>
+      <c r="I828" s="7"/>
     </row>
     <row r="829" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D829" s="11"/>
-      <c r="I829" s="6"/>
+      <c r="I829" s="7"/>
     </row>
     <row r="830" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D830" s="11"/>
-      <c r="I830" s="6"/>
+      <c r="I830" s="7"/>
     </row>
     <row r="831" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D831" s="11"/>
-      <c r="I831" s="6"/>
+      <c r="I831" s="7"/>
     </row>
     <row r="832" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D832" s="11"/>
-      <c r="I832" s="6"/>
+      <c r="I832" s="7"/>
     </row>
     <row r="833" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D833" s="11"/>
-      <c r="I833" s="6"/>
+      <c r="I833" s="7"/>
     </row>
     <row r="834" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D834" s="11"/>
-      <c r="I834" s="6"/>
+      <c r="I834" s="7"/>
     </row>
     <row r="835" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D835" s="11"/>
-      <c r="I835" s="6"/>
+      <c r="I835" s="7"/>
     </row>
     <row r="836" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D836" s="11"/>
-      <c r="I836" s="6"/>
+      <c r="I836" s="7"/>
     </row>
     <row r="837" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D837" s="11"/>
-      <c r="I837" s="6"/>
+      <c r="I837" s="7"/>
     </row>
     <row r="838" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D838" s="11"/>
-      <c r="I838" s="6"/>
+      <c r="I838" s="7"/>
     </row>
     <row r="839" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D839" s="11"/>
-      <c r="I839" s="6"/>
+      <c r="I839" s="7"/>
     </row>
     <row r="840" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D840" s="11"/>
-      <c r="I840" s="6"/>
+      <c r="I840" s="7"/>
     </row>
     <row r="841" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D841" s="11"/>
-      <c r="I841" s="6"/>
+      <c r="I841" s="7"/>
     </row>
     <row r="842" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D842" s="11"/>
-      <c r="I842" s="6"/>
+      <c r="I842" s="7"/>
     </row>
     <row r="843" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D843" s="11"/>
-      <c r="I843" s="6"/>
+      <c r="I843" s="7"/>
     </row>
     <row r="844" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D844" s="11"/>
-      <c r="I844" s="6"/>
+      <c r="I844" s="7"/>
     </row>
     <row r="845" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D845" s="11"/>
-      <c r="I845" s="6"/>
+      <c r="I845" s="7"/>
     </row>
     <row r="846" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D846" s="11"/>
-      <c r="I846" s="6"/>
+      <c r="I846" s="7"/>
     </row>
     <row r="847" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D847" s="11"/>
-      <c r="I847" s="6"/>
+      <c r="I847" s="7"/>
     </row>
     <row r="848" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D848" s="11"/>
-      <c r="I848" s="6"/>
+      <c r="I848" s="7"/>
     </row>
     <row r="849" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D849" s="11"/>
-      <c r="I849" s="6"/>
+      <c r="I849" s="7"/>
     </row>
     <row r="850" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D850" s="11"/>
-      <c r="I850" s="6"/>
+      <c r="I850" s="7"/>
     </row>
     <row r="851" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D851" s="11"/>
-      <c r="I851" s="6"/>
+      <c r="I851" s="7"/>
     </row>
     <row r="852" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D852" s="11"/>
-      <c r="I852" s="6"/>
+      <c r="I852" s="7"/>
     </row>
     <row r="853" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D853" s="11"/>
-      <c r="I853" s="6"/>
+      <c r="I853" s="7"/>
     </row>
     <row r="854" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D854" s="11"/>
-      <c r="I854" s="6"/>
+      <c r="I854" s="7"/>
     </row>
     <row r="855" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D855" s="11"/>
-      <c r="I855" s="6"/>
+      <c r="I855" s="7"/>
     </row>
     <row r="856" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D856" s="11"/>
-      <c r="I856" s="6"/>
+      <c r="I856" s="7"/>
     </row>
     <row r="857" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D857" s="11"/>
-      <c r="I857" s="6"/>
+      <c r="I857" s="7"/>
     </row>
     <row r="858" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D858" s="11"/>
-      <c r="I858" s="6"/>
+      <c r="I858" s="7"/>
     </row>
     <row r="859" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D859" s="11"/>
-      <c r="I859" s="6"/>
+      <c r="I859" s="7"/>
     </row>
     <row r="860" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D860" s="11"/>
-      <c r="I860" s="6"/>
+      <c r="I860" s="7"/>
     </row>
     <row r="861" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D861" s="11"/>
-      <c r="I861" s="6"/>
+      <c r="I861" s="7"/>
     </row>
     <row r="862" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D862" s="11"/>
-      <c r="I862" s="6"/>
+      <c r="I862" s="7"/>
     </row>
     <row r="863" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D863" s="11"/>
-      <c r="I863" s="6"/>
+      <c r="I863" s="7"/>
     </row>
     <row r="864" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D864" s="11"/>
-      <c r="I864" s="6"/>
+      <c r="I864" s="7"/>
     </row>
     <row r="865" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D865" s="11"/>
-      <c r="I865" s="6"/>
+      <c r="I865" s="7"/>
     </row>
     <row r="866" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D866" s="11"/>
-      <c r="I866" s="6"/>
+      <c r="I866" s="7"/>
     </row>
     <row r="867" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D867" s="11"/>
-      <c r="I867" s="6"/>
+      <c r="I867" s="7"/>
     </row>
     <row r="868" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D868" s="11"/>
-      <c r="I868" s="6"/>
+      <c r="I868" s="7"/>
     </row>
     <row r="869" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D869" s="11"/>
-      <c r="I869" s="6"/>
+      <c r="I869" s="7"/>
     </row>
     <row r="870" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D870" s="11"/>
-      <c r="I870" s="6"/>
+      <c r="I870" s="7"/>
     </row>
     <row r="871" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D871" s="11"/>
-      <c r="I871" s="6"/>
+      <c r="I871" s="7"/>
     </row>
     <row r="872" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D872" s="11"/>
-      <c r="I872" s="6"/>
+      <c r="I872" s="7"/>
     </row>
     <row r="873" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D873" s="11"/>
-      <c r="I873" s="6"/>
+      <c r="I873" s="7"/>
     </row>
     <row r="874" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D874" s="11"/>
-      <c r="I874" s="6"/>
+      <c r="I874" s="7"/>
     </row>
     <row r="875" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D875" s="11"/>
-      <c r="I875" s="6"/>
+      <c r="I875" s="7"/>
     </row>
     <row r="876" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D876" s="11"/>
-      <c r="I876" s="6"/>
+      <c r="I876" s="7"/>
     </row>
     <row r="877" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D877" s="11"/>
-      <c r="I877" s="6"/>
+      <c r="I877" s="7"/>
     </row>
     <row r="878" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D878" s="11"/>
-      <c r="I878" s="6"/>
+      <c r="I878" s="7"/>
     </row>
     <row r="879" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D879" s="11"/>
-      <c r="I879" s="6"/>
+      <c r="I879" s="7"/>
     </row>
     <row r="880" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D880" s="11"/>
-      <c r="I880" s="6"/>
+      <c r="I880" s="7"/>
     </row>
     <row r="881" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D881" s="11"/>
-      <c r="I881" s="6"/>
+      <c r="I881" s="7"/>
     </row>
     <row r="882" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D882" s="11"/>
-      <c r="I882" s="6"/>
+      <c r="I882" s="7"/>
     </row>
     <row r="883" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D883" s="11"/>
-      <c r="I883" s="6"/>
+      <c r="I883" s="7"/>
     </row>
     <row r="884" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D884" s="11"/>
-      <c r="I884" s="6"/>
+      <c r="I884" s="7"/>
     </row>
     <row r="885" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D885" s="11"/>
-      <c r="I885" s="6"/>
+      <c r="I885" s="7"/>
     </row>
     <row r="886" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D886" s="11"/>
-      <c r="I886" s="6"/>
+      <c r="I886" s="7"/>
     </row>
     <row r="887" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D887" s="11"/>
-      <c r="I887" s="6"/>
+      <c r="I887" s="7"/>
     </row>
     <row r="888" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D888" s="11"/>
-      <c r="I888" s="6"/>
+      <c r="I888" s="7"/>
     </row>
     <row r="889" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D889" s="11"/>
-      <c r="I889" s="6"/>
+      <c r="I889" s="7"/>
     </row>
     <row r="890" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D890" s="11"/>
-      <c r="I890" s="6"/>
+      <c r="I890" s="7"/>
     </row>
     <row r="891" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D891" s="11"/>
-      <c r="I891" s="6"/>
+      <c r="I891" s="7"/>
     </row>
     <row r="892" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D892" s="11"/>
-      <c r="I892" s="6"/>
+      <c r="I892" s="7"/>
     </row>
     <row r="893" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D893" s="11"/>
-      <c r="I893" s="6"/>
+      <c r="I893" s="7"/>
     </row>
     <row r="894" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D894" s="11"/>
-      <c r="I894" s="6"/>
+      <c r="I894" s="7"/>
     </row>
     <row r="895" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D895" s="11"/>
-      <c r="I895" s="6"/>
+      <c r="I895" s="7"/>
     </row>
     <row r="896" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D896" s="11"/>
-      <c r="I896" s="6"/>
+      <c r="I896" s="7"/>
     </row>
     <row r="897" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D897" s="11"/>
-      <c r="I897" s="6"/>
+      <c r="I897" s="7"/>
     </row>
     <row r="898" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D898" s="11"/>
-      <c r="I898" s="6"/>
+      <c r="I898" s="7"/>
     </row>
     <row r="899" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D899" s="11"/>
-      <c r="I899" s="6"/>
+      <c r="I899" s="7"/>
     </row>
     <row r="900" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D900" s="11"/>
-      <c r="I900" s="6"/>
+      <c r="I900" s="7"/>
     </row>
     <row r="901" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D901" s="11"/>
-      <c r="I901" s="6"/>
+      <c r="I901" s="7"/>
     </row>
     <row r="902" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D902" s="11"/>
-      <c r="I902" s="6"/>
+      <c r="I902" s="7"/>
     </row>
     <row r="903" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D903" s="11"/>
-      <c r="I903" s="6"/>
+      <c r="I903" s="7"/>
     </row>
     <row r="904" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D904" s="11"/>
-      <c r="I904" s="6"/>
+      <c r="I904" s="7"/>
     </row>
     <row r="905" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D905" s="11"/>
-      <c r="I905" s="6"/>
+      <c r="I905" s="7"/>
     </row>
     <row r="906" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D906" s="11"/>
-      <c r="I906" s="6"/>
+      <c r="I906" s="7"/>
     </row>
     <row r="907" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D907" s="11"/>
-      <c r="I907" s="6"/>
+      <c r="I907" s="7"/>
     </row>
     <row r="908" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D908" s="11"/>
-      <c r="I908" s="6"/>
+      <c r="I908" s="7"/>
     </row>
     <row r="909" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D909" s="11"/>
-      <c r="I909" s="6"/>
+      <c r="I909" s="7"/>
     </row>
     <row r="910" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D910" s="11"/>
-      <c r="I910" s="6"/>
+      <c r="I910" s="7"/>
     </row>
     <row r="911" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D911" s="11"/>
-      <c r="I911" s="6"/>
+      <c r="I911" s="7"/>
     </row>
     <row r="912" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D912" s="11"/>
-      <c r="I912" s="6"/>
+      <c r="I912" s="7"/>
     </row>
     <row r="913" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D913" s="11"/>
-      <c r="I913" s="6"/>
+      <c r="I913" s="7"/>
     </row>
     <row r="914" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D914" s="11"/>
-      <c r="I914" s="6"/>
+      <c r="I914" s="7"/>
     </row>
     <row r="915" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D915" s="11"/>
-      <c r="I915" s="6"/>
+      <c r="I915" s="7"/>
     </row>
     <row r="916" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D916" s="11"/>
-      <c r="I916" s="6"/>
+      <c r="I916" s="7"/>
     </row>
     <row r="917" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D917" s="11"/>
-      <c r="I917" s="6"/>
+      <c r="I917" s="7"/>
     </row>
     <row r="918" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D918" s="11"/>
-      <c r="I918" s="6"/>
+      <c r="I918" s="7"/>
     </row>
     <row r="919" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D919" s="11"/>
-      <c r="I919" s="6"/>
+      <c r="I919" s="7"/>
     </row>
     <row r="920" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D920" s="11"/>
-      <c r="I920" s="6"/>
+      <c r="I920" s="7"/>
     </row>
     <row r="921" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D921" s="11"/>
-      <c r="I921" s="6"/>
+      <c r="I921" s="7"/>
     </row>
     <row r="922" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D922" s="11"/>
-      <c r="I922" s="6"/>
+      <c r="I922" s="7"/>
     </row>
     <row r="923" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D923" s="11"/>
-      <c r="I923" s="6"/>
+      <c r="I923" s="7"/>
     </row>
     <row r="924" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D924" s="11"/>
-      <c r="I924" s="6"/>
+      <c r="I924" s="7"/>
     </row>
     <row r="925" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D925" s="11"/>
-      <c r="I925" s="6"/>
+      <c r="I925" s="7"/>
     </row>
     <row r="926" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D926" s="11"/>
-      <c r="I926" s="6"/>
+      <c r="I926" s="7"/>
     </row>
     <row r="927" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D927" s="11"/>
-      <c r="I927" s="6"/>
+      <c r="I927" s="7"/>
     </row>
     <row r="928" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D928" s="11"/>
-      <c r="I928" s="6"/>
+      <c r="I928" s="7"/>
     </row>
     <row r="929" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D929" s="11"/>
-      <c r="I929" s="6"/>
+      <c r="I929" s="7"/>
     </row>
     <row r="930" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D930" s="11"/>
-      <c r="I930" s="6"/>
+      <c r="I930" s="7"/>
     </row>
     <row r="931" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D931" s="11"/>
-      <c r="I931" s="6"/>
+      <c r="I931" s="7"/>
     </row>
     <row r="932" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D932" s="11"/>
-      <c r="I932" s="6"/>
+      <c r="I932" s="7"/>
     </row>
     <row r="933" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D933" s="11"/>
-      <c r="I933" s="6"/>
+      <c r="I933" s="7"/>
     </row>
     <row r="934" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D934" s="11"/>
-      <c r="I934" s="6"/>
+      <c r="I934" s="7"/>
     </row>
     <row r="935" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D935" s="11"/>
-      <c r="I935" s="6"/>
+      <c r="I935" s="7"/>
     </row>
     <row r="936" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D936" s="11"/>
-      <c r="I936" s="6"/>
+      <c r="I936" s="7"/>
     </row>
     <row r="937" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D937" s="11"/>
-      <c r="I937" s="6"/>
+      <c r="I937" s="7"/>
     </row>
     <row r="938" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D938" s="11"/>
-      <c r="I938" s="6"/>
+      <c r="I938" s="7"/>
     </row>
     <row r="939" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D939" s="11"/>
-      <c r="I939" s="6"/>
+      <c r="I939" s="7"/>
     </row>
     <row r="940" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D940" s="11"/>
-      <c r="I940" s="6"/>
+      <c r="I940" s="7"/>
     </row>
     <row r="941" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D941" s="11"/>
-      <c r="I941" s="6"/>
+      <c r="I941" s="7"/>
     </row>
     <row r="942" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D942" s="11"/>
-      <c r="I942" s="6"/>
+      <c r="I942" s="7"/>
     </row>
     <row r="943" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D943" s="11"/>
-      <c r="I943" s="6"/>
+      <c r="I943" s="7"/>
     </row>
     <row r="944" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D944" s="11"/>
-      <c r="I944" s="6"/>
+      <c r="I944" s="7"/>
     </row>
     <row r="945" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D945" s="11"/>
-      <c r="I945" s="6"/>
+      <c r="I945" s="7"/>
     </row>
     <row r="946" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D946" s="11"/>
-      <c r="I946" s="6"/>
+      <c r="I946" s="7"/>
     </row>
     <row r="947" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D947" s="11"/>
-      <c r="I947" s="6"/>
+      <c r="I947" s="7"/>
     </row>
     <row r="948" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D948" s="11"/>
-      <c r="I948" s="6"/>
+      <c r="I948" s="7"/>
     </row>
     <row r="949" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D949" s="11"/>
-      <c r="I949" s="6"/>
+      <c r="I949" s="7"/>
     </row>
     <row r="950" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D950" s="11"/>
-      <c r="I950" s="6"/>
+      <c r="I950" s="7"/>
     </row>
     <row r="951" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D951" s="11"/>
-      <c r="I951" s="6"/>
+      <c r="I951" s="7"/>
     </row>
     <row r="952" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D952" s="11"/>
-      <c r="I952" s="6"/>
+      <c r="I952" s="7"/>
     </row>
     <row r="953" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D953" s="11"/>
-      <c r="I953" s="6"/>
+      <c r="I953" s="7"/>
     </row>
     <row r="954" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D954" s="11"/>
-      <c r="I954" s="6"/>
+      <c r="I954" s="7"/>
     </row>
     <row r="955" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D955" s="11"/>
-      <c r="I955" s="6"/>
+      <c r="I955" s="7"/>
     </row>
     <row r="956" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D956" s="11"/>
-      <c r="I956" s="6"/>
+      <c r="I956" s="7"/>
     </row>
     <row r="957" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D957" s="11"/>
-      <c r="I957" s="6"/>
+      <c r="I957" s="7"/>
     </row>
     <row r="958" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D958" s="11"/>
-      <c r="I958" s="6"/>
+      <c r="I958" s="7"/>
     </row>
     <row r="959" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D959" s="11"/>
-      <c r="I959" s="6"/>
+      <c r="I959" s="7"/>
     </row>
     <row r="960" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D960" s="11"/>
-      <c r="I960" s="6"/>
+      <c r="I960" s="7"/>
     </row>
     <row r="961" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D961" s="11"/>
-      <c r="I961" s="6"/>
+      <c r="I961" s="7"/>
     </row>
     <row r="962" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D962" s="11"/>
-      <c r="I962" s="6"/>
+      <c r="I962" s="7"/>
     </row>
     <row r="963" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D963" s="11"/>
-      <c r="I963" s="6"/>
+      <c r="I963" s="7"/>
     </row>
     <row r="964" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D964" s="11"/>
-      <c r="I964" s="6"/>
+      <c r="I964" s="7"/>
     </row>
     <row r="965" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D965" s="11"/>
-      <c r="I965" s="6"/>
+      <c r="I965" s="7"/>
     </row>
     <row r="966" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D966" s="11"/>
-      <c r="I966" s="6"/>
+      <c r="I966" s="7"/>
     </row>
     <row r="967" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D967" s="11"/>
-      <c r="I967" s="6"/>
+      <c r="I967" s="7"/>
     </row>
     <row r="968" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D968" s="11"/>
-      <c r="I968" s="6"/>
+      <c r="I968" s="7"/>
     </row>
     <row r="969" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D969" s="11"/>
-      <c r="I969" s="6"/>
+      <c r="I969" s="7"/>
     </row>
     <row r="970" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D970" s="11"/>
-      <c r="I970" s="6"/>
+      <c r="I970" s="7"/>
     </row>
     <row r="971" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D971" s="11"/>
-      <c r="I971" s="6"/>
+      <c r="I971" s="7"/>
     </row>
     <row r="972" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D972" s="11"/>
-      <c r="I972" s="6"/>
+      <c r="I972" s="7"/>
     </row>
     <row r="973" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D973" s="11"/>
-      <c r="I973" s="6"/>
+      <c r="I973" s="7"/>
     </row>
     <row r="974" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D974" s="11"/>
-      <c r="I974" s="6"/>
+      <c r="I974" s="7"/>
     </row>
     <row r="975" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D975" s="11"/>
-      <c r="I975" s="6"/>
+      <c r="I975" s="7"/>
     </row>
     <row r="976" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D976" s="11"/>
-      <c r="I976" s="6"/>
+      <c r="I976" s="7"/>
     </row>
     <row r="977" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D977" s="11"/>
-      <c r="I977" s="6"/>
+      <c r="I977" s="7"/>
     </row>
     <row r="978" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D978" s="11"/>
-      <c r="I978" s="6"/>
+      <c r="I978" s="7"/>
     </row>
     <row r="979" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D979" s="11"/>
-      <c r="I979" s="6"/>
+      <c r="I979" s="7"/>
     </row>
     <row r="980" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D980" s="11"/>
-      <c r="I980" s="6"/>
+      <c r="I980" s="7"/>
     </row>
     <row r="981" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D981" s="11"/>
-      <c r="I981" s="6"/>
+      <c r="I981" s="7"/>
     </row>
     <row r="982" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D982" s="11"/>
-      <c r="I982" s="6"/>
+      <c r="I982" s="7"/>
     </row>
     <row r="983" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D983" s="11"/>
-      <c r="I983" s="6"/>
+      <c r="I983" s="7"/>
     </row>
     <row r="984" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D984" s="11"/>
-      <c r="I984" s="6"/>
+      <c r="I984" s="7"/>
     </row>
     <row r="985" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D985" s="11"/>
-      <c r="I985" s="6"/>
+      <c r="I985" s="7"/>
     </row>
     <row r="986" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D986" s="11"/>
-      <c r="I986" s="6"/>
+      <c r="I986" s="7"/>
     </row>
     <row r="987" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D987" s="11"/>
-      <c r="I987" s="6"/>
+      <c r="I987" s="7"/>
     </row>
     <row r="988" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D988" s="11"/>
-      <c r="I988" s="6"/>
+      <c r="I988" s="7"/>
     </row>
     <row r="989" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D989" s="11"/>
-      <c r="I989" s="6"/>
+      <c r="I989" s="7"/>
     </row>
     <row r="990" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D990" s="11"/>
-      <c r="I990" s="6"/>
+      <c r="I990" s="7"/>
     </row>
     <row r="991" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D991" s="11"/>
-      <c r="I991" s="6"/>
+      <c r="I991" s="7"/>
     </row>
     <row r="992" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D992" s="11"/>
-      <c r="I992" s="6"/>
+      <c r="I992" s="7"/>
     </row>
     <row r="993" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D993" s="11"/>
-      <c r="I993" s="6"/>
+      <c r="I993" s="7"/>
     </row>
     <row r="994" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D994" s="11"/>
-      <c r="I994" s="6"/>
+      <c r="I994" s="7"/>
     </row>
     <row r="995" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D995" s="11"/>
-      <c r="I995" s="6"/>
+      <c r="I995" s="7"/>
     </row>
     <row r="996" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D996" s="11"/>
-      <c r="I996" s="6"/>
+      <c r="I996" s="7"/>
     </row>
     <row r="997" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D997" s="11"/>
-      <c r="I997" s="6"/>
+      <c r="I997" s="7"/>
     </row>
     <row r="998" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D998" s="11"/>
-      <c r="I998" s="6"/>
+      <c r="I998" s="7"/>
     </row>
     <row r="999" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D999" s="11"/>
-      <c r="I999" s="6"/>
+      <c r="I999" s="7"/>
     </row>
     <row r="1000" spans="4:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D1000" s="11"/>
-      <c r="I1000" s="6"/>
+      <c r="I1000" s="7"/>
+    </row>
+    <row r="1001" spans="4:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="I1001" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>

</xml_diff>

<commit_message>
Ajuste diciconario de datos
</commit_message>
<xml_diff>
--- a/DiccionarioDatos.xlsx
+++ b/DiccionarioDatos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Documents\USCO\8Semestre\IntegradorIII\documentacionDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8080BD4-06FF-4464-A5DF-D910B52EFFBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4B6AA1-F728-4965-AA5A-27DB96FE0CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,12 +23,11 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Modulo1!$A$1:$K$1016</definedName>
   </definedNames>
   <calcPr calcId="0"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="538">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="539">
   <si>
     <t>Tabla</t>
   </si>
@@ -1643,6 +1642,9 @@
   <si>
     <t>Valor del token de sesión utilizado para identificar y autenticar una sesión activa del usuario en el sistema.</t>
   </si>
+  <si>
+    <t>tipo</t>
+  </si>
 </sst>
 </file>
 
@@ -31775,7 +31777,7 @@
         <v>485</v>
       </c>
       <c r="B84" s="37" t="s">
-        <v>486</v>
+        <v>538</v>
       </c>
       <c r="C84" s="35" t="s">
         <v>487</v>

</xml_diff>

<commit_message>
Ajuste al diciconario de datos
</commit_message>
<xml_diff>
--- a/DiccionarioDatos.xlsx
+++ b/DiccionarioDatos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Documents\USCO\8Semestre\IntegradorIII\documentacionDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4B6AA1-F728-4965-AA5A-27DB96FE0CC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{020E0B91-2068-41A0-AAC1-AA1A9F2A7840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="539">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="540">
   <si>
     <t>Tabla</t>
   </si>
@@ -1592,9 +1592,6 @@
     <t>estado_envio</t>
   </si>
   <si>
-    <t xml:space="preserve"> enum_estado_envio</t>
-  </si>
-  <si>
     <t>Estado del envío de la notificacion</t>
   </si>
   <si>
@@ -1644,6 +1641,12 @@
   </si>
   <si>
     <t>tipo</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> enum_notificaciones_estado_envio</t>
+  </si>
+  <si>
+    <t>Identificador unico de canal de la notificacion</t>
   </si>
 </sst>
 </file>
@@ -2248,7 +2251,7 @@
   <autoFilter ref="A1:K1016" xr:uid="{00000000-0009-0000-0100-000002000000}">
     <filterColumn colId="0">
       <filters>
-        <filter val="tokens"/>
+        <filter val="eventos"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -28949,7 +28952,7 @@
         <v>4</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="C8" s="33" t="s">
         <v>489</v>
@@ -29025,7 +29028,7 @@
         <v>4</v>
       </c>
       <c r="B10" s="33" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="C10" s="33" t="s">
         <v>470</v>
@@ -29339,7 +29342,7 @@
         <v>120</v>
       </c>
       <c r="F18" s="35" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="G18" s="34" t="s">
         <v>122</v>
@@ -29413,7 +29416,7 @@
         <v>120</v>
       </c>
       <c r="F20" s="34" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="G20" s="34" t="s">
         <v>122</v>
@@ -29850,7 +29853,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="32" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="35" t="s">
         <v>450</v>
       </c>
@@ -29888,7 +29891,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="35" t="s">
         <v>450</v>
       </c>
@@ -29917,7 +29920,7 @@
         <v>122</v>
       </c>
       <c r="J33" s="34" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K33" s="36" t="s">
         <v>166</v>
@@ -29926,7 +29929,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="35" t="s">
         <v>450</v>
       </c>
@@ -29964,7 +29967,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="35" t="s">
         <v>450</v>
       </c>
@@ -30002,7 +30005,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="35" t="s">
         <v>450</v>
       </c>
@@ -30040,12 +30043,12 @@
         <v>171</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="35" t="s">
         <v>450</v>
       </c>
       <c r="B37" s="35" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="C37" s="35" t="s">
         <v>451</v>
@@ -30121,7 +30124,7 @@
         <v>433</v>
       </c>
       <c r="B39" s="35" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="C39" s="35" t="s">
         <v>470</v>
@@ -30154,7 +30157,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="35" t="s">
         <v>450</v>
       </c>
@@ -30200,7 +30203,7 @@
         <v>503</v>
       </c>
       <c r="C41" s="35" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D41" s="34" t="s">
         <v>139</v>
@@ -30410,7 +30413,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="49.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="35" t="s">
         <v>450</v>
       </c>
@@ -30446,7 +30449,7 @@
       </c>
       <c r="N47" s="39"/>
     </row>
-    <row r="48" spans="1:14" ht="49.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="35" t="s">
         <v>450</v>
       </c>
@@ -30496,7 +30499,7 @@
       <c r="K49" s="39"/>
       <c r="N49" s="39"/>
     </row>
-    <row r="50" spans="1:14" ht="49.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="35" t="s">
         <v>450</v>
       </c>
@@ -30504,7 +30507,7 @@
         <v>437</v>
       </c>
       <c r="C50" s="35" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="D50" s="35" t="s">
         <v>139</v>
@@ -30528,16 +30531,16 @@
         <v>121</v>
       </c>
       <c r="K50" s="39" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="N50" s="39"/>
     </row>
-    <row r="51" spans="1:14" ht="49.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="35" t="s">
         <v>450</v>
       </c>
       <c r="B51" s="35" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C51" s="35" t="s">
         <v>470</v>
@@ -30564,11 +30567,11 @@
         <v>121</v>
       </c>
       <c r="K51" s="39" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="N51" s="39"/>
     </row>
-    <row r="52" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="35" t="s">
         <v>450</v>
       </c>
@@ -30766,7 +30769,7 @@
         <v>466</v>
       </c>
       <c r="C57" s="35" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="D57" s="34" t="s">
         <v>139</v>
@@ -30804,7 +30807,7 @@
         <v>428</v>
       </c>
       <c r="C58" s="34" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="D58" s="38" t="s">
         <v>172</v>
@@ -31208,7 +31211,7 @@
         <v>121</v>
       </c>
       <c r="K68" s="36" t="s">
-        <v>196</v>
+        <v>539</v>
       </c>
       <c r="N68" s="36" t="s">
         <v>196</v>
@@ -31307,7 +31310,7 @@
         <v>30</v>
       </c>
       <c r="F71" s="35" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="G71" s="35" t="s">
         <v>121</v>
@@ -31322,7 +31325,7 @@
         <v>121</v>
       </c>
       <c r="K71" s="39" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="N71" s="36"/>
     </row>
@@ -31334,7 +31337,7 @@
         <v>520</v>
       </c>
       <c r="C72" s="35" t="s">
-        <v>521</v>
+        <v>538</v>
       </c>
       <c r="D72" s="38" t="s">
         <v>172</v>
@@ -31358,7 +31361,7 @@
         <v>121</v>
       </c>
       <c r="K72" s="39" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="N72" s="36"/>
     </row>
@@ -31736,7 +31739,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="83" spans="1:14" ht="46.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:14" ht="46.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="37" t="s">
         <v>485</v>
       </c>
@@ -31772,12 +31775,12 @@
       </c>
       <c r="N83" s="36"/>
     </row>
-    <row r="84" spans="1:14" ht="39" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:14" ht="39" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="37" t="s">
         <v>485</v>
       </c>
       <c r="B84" s="37" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="C84" s="35" t="s">
         <v>487</v>
@@ -31808,7 +31811,7 @@
       </c>
       <c r="N84" s="36"/>
     </row>
-    <row r="85" spans="1:14" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:14" ht="30.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="37" t="s">
         <v>485</v>
       </c>
@@ -31844,7 +31847,7 @@
       </c>
       <c r="N85" s="36"/>
     </row>
-    <row r="86" spans="1:14" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" ht="30.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="37" t="s">
         <v>485</v>
       </c>
@@ -31876,11 +31879,11 @@
         <v>122</v>
       </c>
       <c r="K86" s="33" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="N86" s="36"/>
     </row>
-    <row r="87" spans="1:14" ht="34.200000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:14" ht="34.200000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="37" t="s">
         <v>485</v>
       </c>
@@ -31916,7 +31919,7 @@
       </c>
       <c r="N87" s="36"/>
     </row>
-    <row r="88" spans="1:14" ht="31.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:14" ht="31.8" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="37" t="s">
         <v>485</v>
       </c>
@@ -37515,7 +37518,7 @@
       <c r="K1015" s="36"/>
       <c r="N1015" s="36"/>
     </row>
-    <row r="1016" spans="1:14" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1016" spans="1:14" ht="12" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="K1016" s="36"/>
       <c r="N1016" s="36"/>
     </row>
@@ -63725,7 +63728,7 @@
     </row>
     <row r="3" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="25" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>431</v>
@@ -63781,7 +63784,7 @@
     </row>
     <row r="7" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="28" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B7" s="28" t="s">
         <v>490</v>

</xml_diff>

<commit_message>
Primera version modelo relacional modulo 9
</commit_message>
<xml_diff>
--- a/DiccionarioDatos.xlsx
+++ b/DiccionarioDatos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\samue\Documents\USCO\8Semestre\IntegradorIII\documentacionDB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{020E0B91-2068-41A0-AAC1-AA1A9F2A7840}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AD59061-FBD2-49C8-AEFD-504D2F9360CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Modulos" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2380" uniqueCount="540">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2382" uniqueCount="542">
   <si>
     <t>Tabla</t>
   </si>
@@ -1643,17 +1643,23 @@
     <t>tipo</t>
   </si>
   <si>
-    <t xml:space="preserve"> enum_notificaciones_estado_envio</t>
+    <t>Identificador unico de canal de la notificacion</t>
   </si>
   <si>
-    <t>Identificador unico de canal de la notificacion</t>
+    <t xml:space="preserve"> enum_notificacion_estado_envio</t>
+  </si>
+  <si>
+    <t>Version</t>
+  </si>
+  <si>
+    <t>2.0.0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1770,6 +1776,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Roboto"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1791,7 +1803,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1917,6 +1929,9 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2235,7 +2250,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Modulos" displayName="Modulos" ref="A1:D1025">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Modulos" displayName="Modulos" ref="A2:D1026">
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Tabla"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Descripción"/>
@@ -2249,9 +2264,9 @@
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Modulo1" displayName="Modulo1" ref="A1:K1016" headerRowDxfId="14" dataDxfId="13" totalsRowDxfId="12">
   <autoFilter ref="A1:K1016" xr:uid="{00000000-0009-0000-0100-000002000000}">
-    <filterColumn colId="0">
+    <filterColumn colId="9">
       <filters>
-        <filter val="eventos"/>
+        <filter val="Si"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -2520,7 +2535,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:W1025"/>
+  <dimension ref="A1:W1026"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.88671875" customWidth="1"/>
@@ -2529,51 +2544,26 @@
     <col min="4" max="4" width="33.33203125" style="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:23" ht="60.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="46" t="s">
+        <v>540</v>
+      </c>
+      <c r="B1" s="46" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="21" t="s">
+      <c r="D2" s="21" t="s">
         <v>3</v>
-      </c>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
-      <c r="I1" s="3"/>
-      <c r="J1" s="3"/>
-      <c r="K1" s="3"/>
-      <c r="L1" s="3"/>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
-      <c r="O1" s="3"/>
-      <c r="P1" s="3"/>
-      <c r="Q1" s="3"/>
-      <c r="R1" s="3"/>
-      <c r="S1" s="3"/>
-      <c r="T1" s="3"/>
-      <c r="U1" s="3"/>
-      <c r="V1" s="3"/>
-      <c r="W1" s="3"/>
-    </row>
-    <row r="2" spans="1:23" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="22" t="s">
-        <v>7</v>
       </c>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
@@ -2595,12 +2585,12 @@
       <c r="V2" s="3"/>
       <c r="W2" s="3"/>
     </row>
-    <row r="3" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:23" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>6</v>
@@ -2630,10 +2620,10 @@
     </row>
     <row r="4" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>6</v>
@@ -2663,13 +2653,13 @@
     </row>
     <row r="5" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D5" s="22" t="s">
         <v>7</v>
@@ -2696,13 +2686,13 @@
     </row>
     <row r="6" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>450</v>
+        <v>12</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D6" s="22" t="s">
         <v>7</v>
@@ -2729,13 +2719,13 @@
     </row>
     <row r="7" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D7" s="22" t="s">
         <v>7</v>
@@ -2762,13 +2752,13 @@
     </row>
     <row r="8" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>19</v>
+        <v>452</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D8" s="22" t="s">
         <v>7</v>
@@ -2795,13 +2785,13 @@
     </row>
     <row r="9" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D9" s="22" t="s">
         <v>7</v>
@@ -2826,15 +2816,15 @@
       <c r="V9" s="3"/>
       <c r="W9" s="3"/>
     </row>
-    <row r="10" spans="1:23" ht="66" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>453</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>22</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D10" s="22" t="s">
         <v>7</v>
@@ -2859,12 +2849,12 @@
       <c r="V10" s="3"/>
       <c r="W10" s="3"/>
     </row>
-    <row r="11" spans="1:23" ht="79.2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:23" ht="66" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="B11" s="27" t="s">
-        <v>478</v>
+        <v>453</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>23</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>6</v>
@@ -2892,15 +2882,15 @@
       <c r="V11" s="3"/>
       <c r="W11" s="3"/>
     </row>
-    <row r="12" spans="1:23" ht="66" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:23" ht="79.2" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
       <c r="B12" s="27" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D12" s="22" t="s">
         <v>7</v>
@@ -2925,15 +2915,15 @@
       <c r="V12" s="3"/>
       <c r="W12" s="3"/>
     </row>
-    <row r="13" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:23" ht="66" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>485</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>512</v>
+        <v>434</v>
+      </c>
+      <c r="B13" s="27" t="s">
+        <v>479</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D13" s="22" t="s">
         <v>7</v>
@@ -2958,15 +2948,15 @@
       <c r="V13" s="3"/>
       <c r="W13" s="3"/>
     </row>
-    <row r="14" spans="1:23" ht="52.8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:23" ht="39.6" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>24</v>
+        <v>485</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>25</v>
+        <v>512</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D14" s="22" t="s">
         <v>7</v>
@@ -2991,18 +2981,18 @@
       <c r="V14" s="3"/>
       <c r="W14" s="3"/>
     </row>
-    <row r="15" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:23" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>27</v>
+        <v>24</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D15" s="22" t="s">
-        <v>28</v>
+        <v>7</v>
       </c>
       <c r="E15" s="3"/>
       <c r="F15" s="3"/>
@@ -3026,13 +3016,13 @@
     </row>
     <row r="16" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="B16" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="B16" s="4" t="s">
         <v>27</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="D16" s="22" t="s">
         <v>28</v>
@@ -3059,13 +3049,13 @@
     </row>
     <row r="17" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="D17" s="22" t="s">
         <v>28</v>
@@ -3092,13 +3082,13 @@
     </row>
     <row r="18" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D18" s="22" t="s">
         <v>28</v>
@@ -3125,10 +3115,10 @@
     </row>
     <row r="19" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>18</v>
@@ -3158,10 +3148,10 @@
     </row>
     <row r="20" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>18</v>
@@ -3191,13 +3181,13 @@
     </row>
     <row r="21" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D21" s="22" t="s">
         <v>28</v>
@@ -3224,13 +3214,13 @@
     </row>
     <row r="22" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D22" s="22" t="s">
         <v>28</v>
@@ -3257,13 +3247,13 @@
     </row>
     <row r="23" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D23" s="22" t="s">
         <v>28</v>
@@ -3290,10 +3280,10 @@
     </row>
     <row r="24" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>6</v>
@@ -3323,13 +3313,13 @@
     </row>
     <row r="25" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D25" s="22" t="s">
         <v>28</v>
@@ -3356,13 +3346,13 @@
     </row>
     <row r="26" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D26" s="22" t="s">
         <v>28</v>
@@ -3389,13 +3379,13 @@
     </row>
     <row r="27" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="D27" s="22" t="s">
         <v>28</v>
@@ -3422,13 +3412,13 @@
     </row>
     <row r="28" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="D28" s="22" t="s">
         <v>28</v>
@@ -3455,13 +3445,13 @@
     </row>
     <row r="29" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D29" s="22" t="s">
         <v>28</v>
@@ -3488,13 +3478,13 @@
     </row>
     <row r="30" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="D30" s="22" t="s">
         <v>28</v>
@@ -3521,13 +3511,13 @@
     </row>
     <row r="31" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="D31" s="22" t="s">
         <v>28</v>
@@ -3554,13 +3544,13 @@
     </row>
     <row r="32" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="D32" s="22" t="s">
         <v>28</v>
@@ -3587,13 +3577,13 @@
     </row>
     <row r="33" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="D33" s="22" t="s">
         <v>28</v>
@@ -3620,13 +3610,13 @@
     </row>
     <row r="34" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="D34" s="22" t="s">
         <v>28</v>
@@ -3653,13 +3643,13 @@
     </row>
     <row r="35" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="D35" s="22" t="s">
         <v>28</v>
@@ -3686,16 +3676,16 @@
     </row>
     <row r="36" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="B36" s="7" t="s">
-        <v>70</v>
+        <v>67</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>68</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>6</v>
       </c>
       <c r="D36" s="22" t="s">
-        <v>71</v>
+        <v>28</v>
       </c>
       <c r="E36" s="3"/>
       <c r="F36" s="3"/>
@@ -3719,13 +3709,13 @@
     </row>
     <row r="37" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="D37" s="22" t="s">
         <v>71</v>
@@ -3752,13 +3742,13 @@
     </row>
     <row r="38" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>76</v>
+        <v>18</v>
       </c>
       <c r="D38" s="22" t="s">
         <v>71</v>
@@ -3785,13 +3775,13 @@
     </row>
     <row r="39" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>18</v>
+        <v>76</v>
       </c>
       <c r="D39" s="22" t="s">
         <v>71</v>
@@ -3818,13 +3808,13 @@
     </row>
     <row r="40" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="D40" s="22" t="s">
         <v>71</v>
@@ -3851,13 +3841,13 @@
     </row>
     <row r="41" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="D41" s="22" t="s">
         <v>71</v>
@@ -3884,10 +3874,10 @@
     </row>
     <row r="42" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B42" s="7" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="C42" s="5" t="s">
         <v>18</v>
@@ -3917,10 +3907,10 @@
     </row>
     <row r="43" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C43" s="5" t="s">
         <v>18</v>
@@ -3950,10 +3940,10 @@
     </row>
     <row r="44" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C44" s="5" t="s">
         <v>18</v>
@@ -3983,13 +3973,13 @@
     </row>
     <row r="45" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="D45" s="22" t="s">
         <v>71</v>
@@ -4016,13 +4006,13 @@
     </row>
     <row r="46" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="D46" s="22" t="s">
         <v>71</v>
@@ -4049,10 +4039,10 @@
     </row>
     <row r="47" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C47" s="5" t="s">
         <v>18</v>
@@ -4082,13 +4072,13 @@
     </row>
     <row r="48" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="D48" s="22" t="s">
         <v>71</v>
@@ -4115,10 +4105,10 @@
     </row>
     <row r="49" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>52</v>
@@ -4148,13 +4138,13 @@
     </row>
     <row r="50" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>6</v>
+        <v>52</v>
       </c>
       <c r="D50" s="22" t="s">
         <v>71</v>
@@ -4181,10 +4171,10 @@
     </row>
     <row r="51" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C51" s="5" t="s">
         <v>6</v>
@@ -4214,13 +4204,13 @@
     </row>
     <row r="52" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>52</v>
+        <v>6</v>
       </c>
       <c r="D52" s="22" t="s">
         <v>71</v>
@@ -4247,13 +4237,13 @@
     </row>
     <row r="53" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>18</v>
+        <v>52</v>
       </c>
       <c r="D53" s="22" t="s">
         <v>71</v>
@@ -4280,13 +4270,13 @@
     </row>
     <row r="54" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>52</v>
+        <v>18</v>
       </c>
       <c r="D54" s="22" t="s">
         <v>71</v>
@@ -4313,13 +4303,13 @@
     </row>
     <row r="55" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>111</v>
+        <v>52</v>
       </c>
       <c r="D55" s="22" t="s">
         <v>71</v>
@@ -4345,10 +4335,18 @@
       <c r="W55" s="3"/>
     </row>
     <row r="56" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="4"/>
-      <c r="B56" s="7"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="23"/>
+      <c r="A56" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B56" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="C56" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="D56" s="22" t="s">
+        <v>71</v>
+      </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3"/>
       <c r="G56" s="3"/>
@@ -4396,7 +4394,7 @@
     </row>
     <row r="58" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4"/>
-      <c r="B58" s="4"/>
+      <c r="B58" s="7"/>
       <c r="C58" s="5"/>
       <c r="D58" s="23"/>
       <c r="E58" s="3"/>
@@ -28573,9 +28571,7 @@
       <c r="A1025" s="4"/>
       <c r="B1025" s="4"/>
       <c r="C1025" s="5"/>
-      <c r="D1025" s="22" t="s">
-        <v>71</v>
-      </c>
+      <c r="D1025" s="23"/>
       <c r="E1025" s="3"/>
       <c r="F1025" s="3"/>
       <c r="G1025" s="3"/>
@@ -28596,63 +28592,90 @@
       <c r="V1025" s="3"/>
       <c r="W1025" s="3"/>
     </row>
+    <row r="1026" spans="1:23" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1026" s="4"/>
+      <c r="B1026" s="4"/>
+      <c r="C1026" s="5"/>
+      <c r="D1026" s="22" t="s">
+        <v>71</v>
+      </c>
+      <c r="E1026" s="3"/>
+      <c r="F1026" s="3"/>
+      <c r="G1026" s="3"/>
+      <c r="H1026" s="3"/>
+      <c r="I1026" s="3"/>
+      <c r="J1026" s="3"/>
+      <c r="K1026" s="3"/>
+      <c r="L1026" s="3"/>
+      <c r="M1026" s="3"/>
+      <c r="N1026" s="3"/>
+      <c r="O1026" s="3"/>
+      <c r="P1026" s="3"/>
+      <c r="Q1026" s="3"/>
+      <c r="R1026" s="3"/>
+      <c r="S1026" s="3"/>
+      <c r="T1026" s="3"/>
+      <c r="U1026" s="3"/>
+      <c r="V1026" s="3"/>
+      <c r="W1026" s="3"/>
+    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D2" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="D3" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="D4" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="D5" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="D6" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="D7" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="D8" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="D9" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="D10" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="D14" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="D15" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="D16" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="D17" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="D18" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="D19" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="D20" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="D21" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="D22" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="D23" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="D24" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="D25" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="D26" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="D27" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="D28" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="D29" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="D30" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="D31" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="D32" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="D33" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="D34" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="D35" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="D36" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="D37" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="D38" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="D39" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="D40" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="D41" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="D42" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="D43" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="D44" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="D45" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="D46" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="D47" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="D48" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="D49" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="D50" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="D51" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="D52" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="D53" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="D54" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="D55" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="D1025" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="D11" location="Modulo1!A1" display="Modulo 1" xr:uid="{62DD4255-4A35-4B22-ADDA-775BB61C6DB0}"/>
-    <hyperlink ref="D12" location="Modulo1!A1" display="Modulo 1" xr:uid="{F7765F97-835C-4AD2-BB4B-4F5C773F35F9}"/>
-    <hyperlink ref="D13" location="Modulo1!A1" display="Modulo 1" xr:uid="{31589241-E646-4B70-A6A1-0CD8DCE8C7CD}"/>
+    <hyperlink ref="D3" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="D4" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="D5" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="D6" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="D7" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="D8" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="D9" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="D10" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="D11" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="D15" location="Modulo1!A1" display="Modulo 1" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="D16" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="D17" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="D18" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="D19" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="D20" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="D21" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="D22" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="D23" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="D24" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="D25" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="D26" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="D27" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="D28" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="D29" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="D30" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="D31" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="D32" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="D33" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="D34" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="D35" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="D36" location="'Modulo 9'!A1" display="Modulo 9" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="D37" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="D38" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="D39" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="D40" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="D41" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="D42" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="D43" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="D44" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="D45" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="D46" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="D47" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="D48" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="D49" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="D50" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="D51" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="D52" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="D53" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="D54" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="D55" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="D56" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="D1026" location="'Modulo 2'!A1" display="Modulo 2" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="D12" location="Modulo1!A1" display="Modulo 1" xr:uid="{62DD4255-4A35-4B22-ADDA-775BB61C6DB0}"/>
+    <hyperlink ref="D13" location="Modulo1!A1" display="Modulo 1" xr:uid="{F7765F97-835C-4AD2-BB4B-4F5C773F35F9}"/>
+    <hyperlink ref="D14" location="Modulo1!A1" display="Modulo 1" xr:uid="{31589241-E646-4B70-A6A1-0CD8DCE8C7CD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
@@ -28719,7 +28742,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="2" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="33" t="s">
         <v>4</v>
       </c>
@@ -28795,7 +28818,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="33" t="s">
         <v>4</v>
       </c>
@@ -28985,7 +29008,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="33" t="s">
         <v>4</v>
       </c>
@@ -29211,7 +29234,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="15" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="33" t="s">
         <v>10</v>
       </c>
@@ -29249,7 +29272,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="16" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="33" t="s">
         <v>10</v>
       </c>
@@ -29437,7 +29460,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="21" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="33" t="s">
         <v>12</v>
       </c>
@@ -29475,7 +29498,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="22" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="33" t="s">
         <v>12</v>
       </c>
@@ -29551,7 +29574,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="24" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="33" t="s">
         <v>8</v>
       </c>
@@ -29589,7 +29612,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="25" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="33" t="s">
         <v>8</v>
       </c>
@@ -29815,7 +29838,7 @@
       </c>
       <c r="N30" s="36"/>
     </row>
-    <row r="31" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="33" t="s">
         <v>8</v>
       </c>
@@ -29891,7 +29914,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="33" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="35" t="s">
         <v>450</v>
       </c>
@@ -29929,7 +29952,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="34" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="35" t="s">
         <v>450</v>
       </c>
@@ -29967,7 +29990,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="35" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="35" t="s">
         <v>450</v>
       </c>
@@ -30005,7 +30028,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="36" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="35" t="s">
         <v>450</v>
       </c>
@@ -30043,7 +30066,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="37" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="35" t="s">
         <v>450</v>
       </c>
@@ -30157,7 +30180,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="40" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="35" t="s">
         <v>450</v>
       </c>
@@ -30375,7 +30398,7 @@
       </c>
       <c r="N45" s="39"/>
     </row>
-    <row r="46" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="35" t="s">
         <v>433</v>
       </c>
@@ -30413,7 +30436,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="47" spans="1:14" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:14" ht="49.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="35" t="s">
         <v>450</v>
       </c>
@@ -30449,7 +30472,7 @@
       </c>
       <c r="N47" s="39"/>
     </row>
-    <row r="48" spans="1:14" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:14" ht="49.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="35" t="s">
         <v>450</v>
       </c>
@@ -30499,7 +30522,7 @@
       <c r="K49" s="39"/>
       <c r="N49" s="39"/>
     </row>
-    <row r="50" spans="1:14" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:14" ht="49.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="35" t="s">
         <v>450</v>
       </c>
@@ -30535,7 +30558,7 @@
       </c>
       <c r="N50" s="39"/>
     </row>
-    <row r="51" spans="1:14" ht="49.2" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:14" ht="49.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="35" t="s">
         <v>450</v>
       </c>
@@ -30571,7 +30594,7 @@
       </c>
       <c r="N51" s="39"/>
     </row>
-    <row r="52" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="35" t="s">
         <v>450</v>
       </c>
@@ -30609,7 +30632,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="53" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="35" t="s">
         <v>452</v>
       </c>
@@ -30647,7 +30670,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="54" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="35" t="s">
         <v>452</v>
       </c>
@@ -30723,7 +30746,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="56" spans="1:14" ht="35.4" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:14" ht="35.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="35" t="s">
         <v>453</v>
       </c>
@@ -30951,7 +30974,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="62" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="35" t="s">
         <v>24</v>
       </c>
@@ -30989,7 +31012,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="63" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="35" t="s">
         <v>24</v>
       </c>
@@ -31065,7 +31088,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="65" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="33" t="s">
         <v>19</v>
       </c>
@@ -31211,7 +31234,7 @@
         <v>121</v>
       </c>
       <c r="K68" s="36" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="N68" s="36" t="s">
         <v>196</v>
@@ -31337,7 +31360,7 @@
         <v>520</v>
       </c>
       <c r="C72" s="35" t="s">
-        <v>538</v>
+        <v>539</v>
       </c>
       <c r="D72" s="38" t="s">
         <v>172</v>
@@ -31403,7 +31426,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="74" spans="1:14" ht="34.950000000000003" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:14" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="35" t="s">
         <v>468</v>
       </c>
@@ -31517,7 +31540,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="77" spans="1:14" ht="19.2" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:14" ht="19.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="32" t="s">
         <v>434</v>
       </c>
@@ -31555,7 +31578,7 @@
         <v>441</v>
       </c>
     </row>
-    <row r="78" spans="1:14" ht="28.8" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:14" ht="28.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="32" t="s">
         <v>434</v>
       </c>
@@ -31847,7 +31870,7 @@
       </c>
       <c r="N85" s="36"/>
     </row>
-    <row r="86" spans="1:14" ht="30.6" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:14" ht="30.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="37" t="s">
         <v>485</v>
       </c>

</xml_diff>